<commit_message>
Version 0.6 - Add photo import workflow and project roadmap
</commit_message>
<xml_diff>
--- a/travelogue/data/Travelogue Data.xlsx
+++ b/travelogue/data/Travelogue Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gscott/Travelogue/travelogue/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9139991-4036-4C47-9508-A1A264E83FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A262967-3D33-D847-AF58-E1953B71E26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="1800" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
+    <workbookView xWindow="0" yWindow="1800" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="156">
   <si>
     <t>Train</t>
   </si>
@@ -498,6 +498,18 @@
   </si>
   <si>
     <t>Rothenberg ob der Tauber</t>
+  </si>
+  <si>
+    <t>Highlight</t>
+  </si>
+  <si>
+    <t>Highlight Title</t>
+  </si>
+  <si>
+    <t>Highlught Note</t>
+  </si>
+  <si>
+    <t>Photo</t>
   </si>
 </sst>
 </file>
@@ -555,23 +567,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yy"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -587,13 +605,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:O46" totalsRowShown="0">
-  <autoFilter ref="C6:O46" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
-  <tableColumns count="13">
-    <tableColumn id="16" xr3:uid="{B7B8133A-8A6E-4EA5-B294-9E2634108185}" name="Trip ID" dataCellStyle="Good"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:S46" totalsRowShown="0">
+  <autoFilter ref="C6:S46" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
+  <tableColumns count="17">
+    <tableColumn id="16" xr3:uid="{B7B8133A-8A6E-4EA5-B294-9E2634108185}" name="Trip ID"/>
     <tableColumn id="1" xr3:uid="{21A3BC19-512C-634F-86B1-18BDC46CFC75}" name="Trip Title"/>
-    <tableColumn id="2" xr3:uid="{BBBE16A1-D09A-4AE1-8F63-8AFDBF217A9F}" name="Start Date" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{E56FF79B-67A8-4495-BE75-8ABC52E5DC1B}" name="End Date" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{BBBE16A1-D09A-4AE1-8F63-8AFDBF217A9F}" name="Start Date" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{E56FF79B-67A8-4495-BE75-8ABC52E5DC1B}" name="End Date" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{085DA54F-08D7-43B8-B0F4-A47955988CBE}" name="Stops"/>
     <tableColumn id="6" xr3:uid="{A38BA83E-4DBF-4DF4-A909-AA3FB3895BF0}" name="Travel Mode"/>
     <tableColumn id="9" xr3:uid="{4DDEA34E-33EA-4A45-A476-B019C92EF7D1}" name="Category"/>
@@ -603,6 +621,10 @@
     <tableColumn id="10" xr3:uid="{EE9B6364-822C-5044-A802-8D0A47DDDCF0}" name="Favorite"/>
     <tableColumn id="11" xr3:uid="{1A0019D0-FB38-3E47-B142-4DCA953885B9}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FDE8B4F8-6186-E445-887C-E336131FF0FB}" name="Public"/>
+    <tableColumn id="13" xr3:uid="{C973B6AD-C4FE-B340-A1BA-AFD890F06300}" name="Highlight" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{F0452C82-0D3D-B047-9111-289C96C71818}" name="Highlight Title" dataDxfId="0"/>
+    <tableColumn id="15" xr3:uid="{0E9D489D-AC48-AE4F-951A-6BF76F81E72F}" name="Highlught Note"/>
+    <tableColumn id="17" xr3:uid="{5E3B0C82-CFC4-354A-A772-91DB57E2EF89}" name="Photo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -928,7 +950,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="C2:Q54"/>
+  <dimension ref="C2:S54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="11.5" customWidth="1"/>
@@ -936,39 +958,40 @@
     <col min="5" max="5" width="11.5" customWidth="1"/>
     <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="79.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="24" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.1640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.1640625" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="24" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" style="5" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="48.1640625" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="0" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="10" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" hidden="1" customWidth="1"/>
     <col min="16" max="17" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:17" ht="27" x14ac:dyDescent="0.35">
-      <c r="C2" s="5" t="s">
+    <row r="2" spans="3:19" ht="27" x14ac:dyDescent="0.35">
+      <c r="C2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-    </row>
-    <row r="3" spans="3:17" x14ac:dyDescent="0.2">
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="3:19" x14ac:dyDescent="0.2">
       <c r="G3" s="4"/>
       <c r="H3" s="3"/>
       <c r="L3" s="2"/>
       <c r="N3" s="2"/>
       <c r="P3" s="2"/>
     </row>
-    <row r="4" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="3:19" x14ac:dyDescent="0.2">
       <c r="L4" s="2"/>
     </row>
-    <row r="6" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>80</v>
       </c>
@@ -993,7 +1016,7 @@
       <c r="J6" t="s">
         <v>123</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="5" t="s">
         <v>124</v>
       </c>
       <c r="L6" t="s">
@@ -1008,8 +1031,20 @@
       <c r="O6" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="7" spans="3:17" x14ac:dyDescent="0.2">
+      <c r="P6" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>153</v>
+      </c>
+      <c r="R6" t="s">
+        <v>154</v>
+      </c>
+      <c r="S6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>81</v>
       </c>
@@ -1031,7 +1066,7 @@
       <c r="I7" t="s">
         <v>137</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="5">
         <v>2</v>
       </c>
       <c r="L7" t="s">
@@ -1049,7 +1084,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="2"/>
     </row>
-    <row r="8" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
         <v>82</v>
       </c>
@@ -1071,7 +1106,7 @@
       <c r="I8" t="s">
         <v>137</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="5">
         <v>2</v>
       </c>
       <c r="L8" t="s">
@@ -1089,7 +1124,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="2"/>
     </row>
-    <row r="9" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C9" t="s">
         <v>83</v>
       </c>
@@ -1111,7 +1146,7 @@
       <c r="I9" t="s">
         <v>133</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="5">
         <v>6</v>
       </c>
       <c r="L9" t="s">
@@ -1129,7 +1164,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="2"/>
     </row>
-    <row r="10" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C10" t="s">
         <v>84</v>
       </c>
@@ -1151,7 +1186,7 @@
       <c r="I10" t="s">
         <v>134</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="5">
         <v>2</v>
       </c>
       <c r="L10" t="s">
@@ -1169,7 +1204,7 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="2"/>
     </row>
-    <row r="11" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
         <v>85</v>
       </c>
@@ -1191,7 +1226,7 @@
       <c r="I11" t="s">
         <v>134</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="5">
         <v>2</v>
       </c>
       <c r="L11" t="s">
@@ -1209,7 +1244,7 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="2"/>
     </row>
-    <row r="12" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
         <v>86</v>
       </c>
@@ -1231,7 +1266,7 @@
       <c r="I12" t="s">
         <v>138</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="5">
         <v>2</v>
       </c>
       <c r="L12" t="s">
@@ -1249,7 +1284,7 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="2"/>
     </row>
-    <row r="13" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C13" t="s">
         <v>87</v>
       </c>
@@ -1271,7 +1306,7 @@
       <c r="I13" t="s">
         <v>136</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="5">
         <v>2</v>
       </c>
       <c r="L13" t="s">
@@ -1289,7 +1324,7 @@
       <c r="P13" s="1"/>
       <c r="Q13" s="2"/>
     </row>
-    <row r="14" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C14" t="s">
         <v>88</v>
       </c>
@@ -1311,7 +1346,7 @@
       <c r="I14" t="s">
         <v>135</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="5">
         <v>2</v>
       </c>
       <c r="L14" t="s">
@@ -1329,7 +1364,7 @@
       <c r="P14" s="1"/>
       <c r="Q14" s="2"/>
     </row>
-    <row r="15" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C15" t="s">
         <v>89</v>
       </c>
@@ -1351,7 +1386,7 @@
       <c r="I15" t="s">
         <v>135</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="5">
         <v>4</v>
       </c>
       <c r="L15" t="s">
@@ -1369,7 +1404,7 @@
       <c r="P15" s="1"/>
       <c r="Q15" s="2"/>
     </row>
-    <row r="16" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C16" t="s">
         <v>90</v>
       </c>
@@ -1391,7 +1426,7 @@
       <c r="I16" t="s">
         <v>133</v>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="5">
         <v>3</v>
       </c>
       <c r="L16" t="s">
@@ -1431,7 +1466,7 @@
       <c r="I17" t="s">
         <v>132</v>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="5">
         <v>2</v>
       </c>
       <c r="L17" t="s">
@@ -1471,7 +1506,7 @@
       <c r="I18" t="s">
         <v>136</v>
       </c>
-      <c r="K18" s="6">
+      <c r="K18" s="5">
         <v>7</v>
       </c>
       <c r="L18" t="s">
@@ -1511,7 +1546,7 @@
       <c r="I19" t="s">
         <v>138</v>
       </c>
-      <c r="K19" s="6">
+      <c r="K19" s="5">
         <v>2</v>
       </c>
       <c r="L19" t="s">
@@ -1551,7 +1586,7 @@
       <c r="I20" t="s">
         <v>136</v>
       </c>
-      <c r="K20" s="6">
+      <c r="K20" s="5">
         <v>4</v>
       </c>
       <c r="L20" t="s">
@@ -1591,7 +1626,7 @@
       <c r="I21" t="s">
         <v>137</v>
       </c>
-      <c r="K21" s="6">
+      <c r="K21" s="5">
         <v>4</v>
       </c>
       <c r="L21" t="s">
@@ -1631,7 +1666,7 @@
       <c r="I22" t="s">
         <v>138</v>
       </c>
-      <c r="K22" s="6">
+      <c r="K22" s="5">
         <v>6</v>
       </c>
       <c r="L22" t="s">
@@ -1671,7 +1706,7 @@
       <c r="I23" t="s">
         <v>133</v>
       </c>
-      <c r="K23" s="6">
+      <c r="K23" s="5">
         <v>2</v>
       </c>
       <c r="L23" t="s">
@@ -1711,7 +1746,7 @@
       <c r="I24" t="s">
         <v>139</v>
       </c>
-      <c r="K24" s="6">
+      <c r="K24" s="5">
         <v>4</v>
       </c>
       <c r="L24" t="s">
@@ -1751,7 +1786,7 @@
       <c r="I25" t="s">
         <v>7</v>
       </c>
-      <c r="K25" s="6">
+      <c r="K25" s="5">
         <v>2</v>
       </c>
       <c r="L25" t="s">
@@ -1791,7 +1826,7 @@
       <c r="I26" t="s">
         <v>133</v>
       </c>
-      <c r="K26" s="6">
+      <c r="K26" s="5">
         <v>4</v>
       </c>
       <c r="L26" t="s">
@@ -1829,7 +1864,7 @@
       <c r="I27" t="s">
         <v>138</v>
       </c>
-      <c r="K27" s="6">
+      <c r="K27" s="5">
         <v>2</v>
       </c>
       <c r="L27" t="s">
@@ -1869,7 +1904,7 @@
       <c r="I28" t="s">
         <v>134</v>
       </c>
-      <c r="K28" s="6">
+      <c r="K28" s="5">
         <v>2</v>
       </c>
       <c r="L28" t="s">
@@ -1909,7 +1944,7 @@
       <c r="I29" t="s">
         <v>141</v>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="5">
         <v>2</v>
       </c>
       <c r="L29" t="s">
@@ -1949,7 +1984,7 @@
       <c r="I30" t="s">
         <v>134</v>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="5">
         <v>4</v>
       </c>
       <c r="L30" t="s">
@@ -1989,7 +2024,7 @@
       <c r="I31" t="s">
         <v>134</v>
       </c>
-      <c r="K31" s="6">
+      <c r="K31" s="5">
         <v>2</v>
       </c>
       <c r="L31" t="s">
@@ -2029,7 +2064,7 @@
       <c r="I32" t="s">
         <v>134</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K32" s="5">
         <v>2</v>
       </c>
       <c r="L32" t="s">
@@ -2069,7 +2104,7 @@
       <c r="I33" t="s">
         <v>138</v>
       </c>
-      <c r="K33" s="6">
+      <c r="K33" s="5">
         <v>4</v>
       </c>
       <c r="L33" t="s">
@@ -2109,7 +2144,7 @@
       <c r="I34" t="s">
         <v>136</v>
       </c>
-      <c r="K34" s="6">
+      <c r="K34" s="5">
         <v>4</v>
       </c>
       <c r="L34" t="s">
@@ -2149,7 +2184,7 @@
       <c r="I35" t="s">
         <v>138</v>
       </c>
-      <c r="K35" s="6">
+      <c r="K35" s="5">
         <v>5</v>
       </c>
       <c r="L35" t="s">
@@ -2189,7 +2224,7 @@
       <c r="I36" t="s">
         <v>135</v>
       </c>
-      <c r="K36" s="6">
+      <c r="K36" s="5">
         <v>2</v>
       </c>
       <c r="L36" t="s">
@@ -2229,7 +2264,7 @@
       <c r="I37" t="s">
         <v>133</v>
       </c>
-      <c r="K37" s="6">
+      <c r="K37" s="5">
         <v>4</v>
       </c>
       <c r="L37" t="s">
@@ -2269,7 +2304,7 @@
       <c r="I38" t="s">
         <v>132</v>
       </c>
-      <c r="K38" s="6">
+      <c r="K38" s="5">
         <v>2</v>
       </c>
       <c r="L38" t="s">
@@ -2309,7 +2344,7 @@
       <c r="I39" t="s">
         <v>136</v>
       </c>
-      <c r="K39" s="6">
+      <c r="K39" s="5">
         <v>2</v>
       </c>
       <c r="L39" t="s">
@@ -2349,7 +2384,7 @@
       <c r="I40" t="s">
         <v>132</v>
       </c>
-      <c r="K40" s="6">
+      <c r="K40" s="5">
         <v>2</v>
       </c>
       <c r="L40" t="s">
@@ -2389,7 +2424,7 @@
       <c r="I41" t="s">
         <v>139</v>
       </c>
-      <c r="K41" s="6">
+      <c r="K41" s="5">
         <v>2</v>
       </c>
       <c r="L41" t="s">
@@ -2429,7 +2464,7 @@
       <c r="I42" t="s">
         <v>136</v>
       </c>
-      <c r="K42" s="6">
+      <c r="K42" s="5">
         <v>2</v>
       </c>
       <c r="L42" t="s">
@@ -2469,7 +2504,7 @@
       <c r="I43" t="s">
         <v>136</v>
       </c>
-      <c r="K43" s="6">
+      <c r="K43" s="5">
         <v>2</v>
       </c>
       <c r="L43" t="s">
@@ -2509,7 +2544,7 @@
       <c r="I44" t="s">
         <v>133</v>
       </c>
-      <c r="K44" s="6">
+      <c r="K44" s="5">
         <v>6</v>
       </c>
       <c r="L44" t="s">
@@ -2549,7 +2584,7 @@
       <c r="I45" t="s">
         <v>138</v>
       </c>
-      <c r="K45" s="6">
+      <c r="K45" s="5">
         <v>2</v>
       </c>
       <c r="L45" t="s">
@@ -2589,7 +2624,7 @@
       <c r="I46" t="s">
         <v>137</v>
       </c>
-      <c r="K46" s="6">
+      <c r="K46" s="5">
         <v>4</v>
       </c>
       <c r="L46" t="s">

</xml_diff>

<commit_message>
Version 0.7 - Add hero photo and curated journey highlights
</commit_message>
<xml_diff>
--- a/travelogue/data/Travelogue Data.xlsx
+++ b/travelogue/data/Travelogue Data.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gscott/Travelogue/travelogue/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A262967-3D33-D847-AF58-E1953B71E26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AEF414-757C-9944-8334-1E6C6B8A45BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1800" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
+    <workbookView xWindow="180" yWindow="1920" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_MailAutoSig" localSheetId="0">'Sheet1 (2)'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1 (2)'!$C$2:$J$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1 (2)'!$C$2:$J$40</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="204">
   <si>
     <t>Train</t>
   </si>
@@ -125,9 +125,6 @@
     <t>Missing</t>
   </si>
   <si>
-    <t>Nuremberg</t>
-  </si>
-  <si>
     <t>Rhine Mothers Day</t>
   </si>
   <si>
@@ -419,12 +416,6 @@
     <t>Borders Crossed</t>
   </si>
   <si>
-    <t>Heidelbergs</t>
-  </si>
-  <si>
-    <t>Schwetzingens</t>
-  </si>
-  <si>
     <t>Summary</t>
   </si>
   <si>
@@ -497,19 +488,172 @@
     <t>Luxembourg City, Luxembourg; Porto, Portugal</t>
   </si>
   <si>
-    <t>Rothenberg ob der Tauber</t>
-  </si>
-  <si>
     <t>Highlight</t>
   </si>
   <si>
     <t>Highlight Title</t>
   </si>
   <si>
-    <t>Highlught Note</t>
-  </si>
-  <si>
     <t>Photo</t>
+  </si>
+  <si>
+    <t>TRIP-041</t>
+  </si>
+  <si>
+    <t>TRIP-042</t>
+  </si>
+  <si>
+    <t>TRIP-043</t>
+  </si>
+  <si>
+    <t>Zirndorf, Germany; Nuremberg, Germany; Schwetzingen, Germany</t>
+  </si>
+  <si>
+    <t>Playmobil Fun Park &amp; Nürmberg</t>
+  </si>
+  <si>
+    <t>Rothenburg ob der Tauber, Germany</t>
+  </si>
+  <si>
+    <t>Rothenburg ob der Tauber</t>
+  </si>
+  <si>
+    <t>Stuttgart, Germany</t>
+  </si>
+  <si>
+    <t>Highlight Note</t>
+  </si>
+  <si>
+    <t>Doing what we came here to do!</t>
+  </si>
+  <si>
+    <t>Even in the cold of January, Paris warms our hearts.</t>
+  </si>
+  <si>
+    <t>The reason why George moved the family!</t>
+  </si>
+  <si>
+    <t>Refreshing swimming, delicious food, unbeatable views</t>
+  </si>
+  <si>
+    <t>Revisiting our favorite honeymoon spot almost 10 years later</t>
+  </si>
+  <si>
+    <t>Walruses for neighbors and 24-hour access to an incredible zoon</t>
+  </si>
+  <si>
+    <t>First Tour de France</t>
+  </si>
+  <si>
+    <t>First Real Trip</t>
+  </si>
+  <si>
+    <t>George's Favorite Birthday</t>
+  </si>
+  <si>
+    <t>Favorite Ski Trip</t>
+  </si>
+  <si>
+    <t>George's "Can't Stop Thinking About" Trip</t>
+  </si>
+  <si>
+    <t>Best Hotel</t>
+  </si>
+  <si>
+    <t>Big Summer Trip</t>
+  </si>
+  <si>
+    <t>Bucket List Country!</t>
+  </si>
+  <si>
+    <t>Christmas Market Trip</t>
+  </si>
+  <si>
+    <t>Featuring a torch-lit walk</t>
+  </si>
+  <si>
+    <t>And a 10th wedding anniversary!</t>
+  </si>
+  <si>
+    <t>Fanciest Livestock</t>
+  </si>
+  <si>
+    <t>Cows with Hats!</t>
+  </si>
+  <si>
+    <t>Most Nostalgic</t>
+  </si>
+  <si>
+    <t>Best Fall Foliage</t>
+  </si>
+  <si>
+    <t>Most Awe-Inspiring</t>
+  </si>
+  <si>
+    <t>Being citizens of the world</t>
+  </si>
+  <si>
+    <t>Best Hidden Gems</t>
+  </si>
+  <si>
+    <t>Get there before the influencers do!</t>
+  </si>
+  <si>
+    <t>Most Provincial</t>
+  </si>
+  <si>
+    <t>Bonjour! Bonjour! Bonjour!</t>
+  </si>
+  <si>
+    <t>Best Mountains</t>
+  </si>
+  <si>
+    <t>Great hikes, food, and views</t>
+  </si>
+  <si>
+    <t>IMG_0562.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_0767.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_2215.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_2901.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_3151.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_4880.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_5170.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_6167.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_6376.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_6803.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_6900.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_7044.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_8523.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_8679.jpeg</t>
+  </si>
+  <si>
+    <t>IMG_9794.jpeg</t>
   </si>
 </sst>
 </file>
@@ -605,8 +749,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:S46" totalsRowShown="0">
-  <autoFilter ref="C6:S46" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:S49" totalsRowShown="0">
+  <autoFilter ref="C6:S49" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C7:S49">
+    <sortCondition ref="C6:C49"/>
+  </sortState>
   <tableColumns count="17">
     <tableColumn id="16" xr3:uid="{B7B8133A-8A6E-4EA5-B294-9E2634108185}" name="Trip ID"/>
     <tableColumn id="1" xr3:uid="{21A3BC19-512C-634F-86B1-18BDC46CFC75}" name="Trip Title"/>
@@ -623,7 +770,7 @@
     <tableColumn id="12" xr3:uid="{FDE8B4F8-6186-E445-887C-E336131FF0FB}" name="Public"/>
     <tableColumn id="13" xr3:uid="{C973B6AD-C4FE-B340-A1BA-AFD890F06300}" name="Highlight" dataDxfId="1"/>
     <tableColumn id="14" xr3:uid="{F0452C82-0D3D-B047-9111-289C96C71818}" name="Highlight Title" dataDxfId="0"/>
-    <tableColumn id="15" xr3:uid="{0E9D489D-AC48-AE4F-951A-6BF76F81E72F}" name="Highlught Note"/>
+    <tableColumn id="15" xr3:uid="{0E9D489D-AC48-AE4F-951A-6BF76F81E72F}" name="Highlight Note"/>
     <tableColumn id="17" xr3:uid="{5E3B0C82-CFC4-354A-A772-91DB57E2EF89}" name="Photo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -966,8 +1113,9 @@
     <col min="13" max="13" width="0" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="10" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="9.33203125" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:19" ht="27" x14ac:dyDescent="0.35">
@@ -993,7 +1141,7 @@
     </row>
     <row r="6" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -1014,42 +1162,42 @@
         <v>18</v>
       </c>
       <c r="J6" t="s">
+        <v>122</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="L6" t="s">
         <v>124</v>
       </c>
-      <c r="L6" t="s">
-        <v>127</v>
-      </c>
       <c r="M6" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="N6" t="s">
         <v>8</v>
       </c>
       <c r="O6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="P6" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="Q6" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="R6" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="S6" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E7" s="1">
         <v>45535</v>
@@ -1064,32 +1212,34 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="K7" s="5">
         <v>2</v>
       </c>
       <c r="L7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M7" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N7" t="s">
         <v>2</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P7" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q7" s="2"/>
     </row>
     <row r="8" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E8" s="1">
         <v>45556</v>
@@ -1098,38 +1248,40 @@
         <v>45556</v>
       </c>
       <c r="G8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H8" t="s">
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="K8" s="5">
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M8" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N8" t="s">
         <v>2</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P8" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q8" s="2"/>
     </row>
     <row r="9" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E9" s="1">
         <v>45592</v>
@@ -1138,38 +1290,48 @@
         <v>45595</v>
       </c>
       <c r="G9" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="H9" t="s">
         <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K9" s="5">
         <v>6</v>
       </c>
       <c r="L9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N9" t="s">
         <v>2</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="2"/>
+        <v>139</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="R9" t="s">
+        <v>160</v>
+      </c>
+      <c r="S9" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="10" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E10" s="1">
         <v>45640</v>
@@ -1184,32 +1346,34 @@
         <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="K10" s="5">
         <v>2</v>
       </c>
       <c r="L10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="M10" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N10" t="s">
         <v>2</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P10" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q10" s="2"/>
     </row>
     <row r="11" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E11" s="1">
         <v>45654</v>
@@ -1224,32 +1388,34 @@
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="K11" s="5">
         <v>2</v>
       </c>
       <c r="L11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="N11" t="s">
         <v>2</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P11" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q11" s="2"/>
     </row>
     <row r="12" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E12" s="1">
         <v>45667</v>
@@ -1264,32 +1430,42 @@
         <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K12" s="5">
         <v>2</v>
       </c>
       <c r="L12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M12" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N12" t="s">
         <v>2</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="2"/>
+        <v>139</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="R12" t="s">
+        <v>161</v>
+      </c>
+      <c r="S12" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="13" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E13" s="1">
         <v>45674</v>
@@ -1304,32 +1480,34 @@
         <v>3</v>
       </c>
       <c r="I13" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="K13" s="5">
         <v>2</v>
       </c>
       <c r="L13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="M13" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N13" t="s">
         <v>2</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P13" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q13" s="2"/>
     </row>
     <row r="14" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E14" s="1">
         <v>45705</v>
@@ -1338,38 +1516,40 @@
         <v>45705</v>
       </c>
       <c r="G14" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H14" t="s">
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K14" s="5">
         <v>2</v>
       </c>
       <c r="L14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M14" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N14" t="s">
         <v>2</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P14" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q14" s="2"/>
     </row>
     <row r="15" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E15" s="1">
         <v>45711</v>
@@ -1384,29 +1564,39 @@
         <v>1</v>
       </c>
       <c r="I15" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K15" s="5">
         <v>4</v>
       </c>
       <c r="L15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M15" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N15" t="s">
         <v>2</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="2"/>
+        <v>139</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="R15" t="s">
+        <v>162</v>
+      </c>
+      <c r="S15" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="16" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -1418,13 +1608,13 @@
         <v>45768</v>
       </c>
       <c r="G16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H16" t="s">
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K16" s="5">
         <v>3</v>
@@ -1433,20 +1623,22 @@
         <v>11</v>
       </c>
       <c r="M16" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N16" t="s">
         <v>2</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P16" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q16" s="2"/>
     </row>
-    <row r="17" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
@@ -1464,7 +1656,7 @@
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K17" s="5">
         <v>2</v>
@@ -1473,20 +1665,22 @@
         <v>12</v>
       </c>
       <c r="M17" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N17" t="s">
         <v>2</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P17" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q17" s="2"/>
     </row>
-    <row r="18" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D18" t="s">
         <v>13</v>
@@ -1498,13 +1692,13 @@
         <v>45809</v>
       </c>
       <c r="G18" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H18" t="s">
         <v>1</v>
       </c>
       <c r="I18" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="K18" s="5">
         <v>7</v>
@@ -1513,23 +1707,33 @@
         <v>13</v>
       </c>
       <c r="M18" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N18" t="s">
         <v>2</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="2"/>
-    </row>
-    <row r="19" spans="3:17" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q18" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="R18" t="s">
+        <v>163</v>
+      </c>
+      <c r="S18" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E19" s="1">
         <v>45814</v>
@@ -1538,35 +1742,45 @@
         <v>45817</v>
       </c>
       <c r="G19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H19" t="s">
         <v>3</v>
       </c>
       <c r="I19" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K19" s="5">
         <v>2</v>
       </c>
       <c r="L19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="M19" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N19" t="s">
         <v>2</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="2"/>
-    </row>
-    <row r="20" spans="3:17" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q19" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="R19" t="s">
+        <v>164</v>
+      </c>
+      <c r="S19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D20" t="s">
         <v>14</v>
@@ -1578,13 +1792,13 @@
         <v>45844</v>
       </c>
       <c r="G20" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H20" t="s">
         <v>1</v>
       </c>
       <c r="I20" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="K20" s="5">
         <v>4</v>
@@ -1593,20 +1807,22 @@
         <v>14</v>
       </c>
       <c r="M20" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N20" t="s">
         <v>2</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P20" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P20" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q20" s="2"/>
     </row>
-    <row r="21" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D21" t="s">
         <v>15</v>
@@ -1618,13 +1834,13 @@
         <v>45857</v>
       </c>
       <c r="G21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H21" t="s">
         <v>1</v>
       </c>
       <c r="I21" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="K21" s="5">
         <v>4</v>
@@ -1633,20 +1849,30 @@
         <v>15</v>
       </c>
       <c r="M21" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N21" t="s">
         <v>2</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="2"/>
-    </row>
-    <row r="22" spans="3:17" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q21" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="R21" t="s">
+        <v>165</v>
+      </c>
+      <c r="S21" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="22" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D22" t="s">
         <v>16</v>
@@ -1658,13 +1884,13 @@
         <v>45865</v>
       </c>
       <c r="G22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H22" t="s">
         <v>1</v>
       </c>
       <c r="I22" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K22" s="5">
         <v>6</v>
@@ -1673,550 +1899,560 @@
         <v>16</v>
       </c>
       <c r="M22" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N22" t="s">
         <v>2</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P22" s="1"/>
-      <c r="Q22" s="2"/>
-    </row>
-    <row r="23" spans="3:17" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q22" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="R22" t="s">
+        <v>176</v>
+      </c>
+      <c r="S22" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="23" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C23" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" t="s">
+        <v>157</v>
+      </c>
+      <c r="E23" s="1">
+        <v>45870</v>
+      </c>
+      <c r="F23" s="1">
+        <v>45872</v>
+      </c>
+      <c r="G23" t="s">
+        <v>156</v>
+      </c>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q23" s="2"/>
+    </row>
+    <row r="24" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C24" t="s">
         <v>97</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D24" t="s">
+        <v>155</v>
+      </c>
+      <c r="E24" s="1">
+        <v>45877</v>
+      </c>
+      <c r="F24" s="1">
+        <v>45879</v>
+      </c>
+      <c r="G24" t="s">
+        <v>154</v>
+      </c>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q24" s="2"/>
+    </row>
+    <row r="25" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C25" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" t="s">
         <v>17</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E25" s="1">
         <v>45885</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F25" s="1">
         <v>45890</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H25" t="s">
+        <v>120</v>
+      </c>
+      <c r="I25" t="s">
+        <v>130</v>
+      </c>
+      <c r="K25" s="5">
+        <v>2</v>
+      </c>
+      <c r="L25" t="s">
+        <v>17</v>
+      </c>
+      <c r="M25" t="s">
+        <v>139</v>
+      </c>
+      <c r="N25" t="s">
+        <v>2</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P25" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q25" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="R25" t="s">
+        <v>173</v>
+      </c>
+      <c r="S25" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="26" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C26" t="s">
+        <v>99</v>
+      </c>
+      <c r="D26" t="s">
+        <v>145</v>
+      </c>
+      <c r="E26" s="1">
+        <v>45905</v>
+      </c>
+      <c r="F26" s="1">
+        <v>45907</v>
+      </c>
+      <c r="G26" t="s">
         <v>33</v>
       </c>
-      <c r="H23" t="s">
-        <v>121</v>
-      </c>
-      <c r="I23" t="s">
-        <v>133</v>
-      </c>
-      <c r="K23" s="5">
-        <v>2</v>
-      </c>
-      <c r="L23" t="s">
-        <v>17</v>
-      </c>
-      <c r="M23" t="s">
-        <v>142</v>
-      </c>
-      <c r="N23" t="s">
-        <v>2</v>
-      </c>
-      <c r="O23" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="2"/>
-    </row>
-    <row r="24" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C24" t="s">
-        <v>98</v>
-      </c>
-      <c r="D24" t="s">
-        <v>148</v>
-      </c>
-      <c r="E24" s="1">
-        <v>45905</v>
-      </c>
-      <c r="F24" s="1">
-        <v>45907</v>
-      </c>
-      <c r="G24" t="s">
-        <v>34</v>
-      </c>
-      <c r="H24" t="s">
-        <v>1</v>
-      </c>
-      <c r="I24" t="s">
-        <v>139</v>
-      </c>
-      <c r="K24" s="5">
-        <v>4</v>
-      </c>
-      <c r="L24" t="s">
-        <v>35</v>
-      </c>
-      <c r="M24" t="s">
-        <v>142</v>
-      </c>
-      <c r="N24" t="s">
-        <v>2</v>
-      </c>
-      <c r="O24" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="2"/>
-    </row>
-    <row r="25" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C25" t="s">
-        <v>99</v>
-      </c>
-      <c r="D25" t="s">
-        <v>36</v>
-      </c>
-      <c r="E25" s="1">
-        <v>45925</v>
-      </c>
-      <c r="F25" s="1">
-        <v>45928</v>
-      </c>
-      <c r="G25" t="s">
-        <v>22</v>
-      </c>
-      <c r="H25" t="s">
-        <v>1</v>
-      </c>
-      <c r="I25" t="s">
-        <v>7</v>
-      </c>
-      <c r="K25" s="5">
-        <v>2</v>
-      </c>
-      <c r="L25" t="s">
-        <v>36</v>
-      </c>
-      <c r="M25" t="s">
-        <v>142</v>
-      </c>
-      <c r="N25" t="s">
-        <v>2</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="2"/>
-    </row>
-    <row r="26" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C26" t="s">
-        <v>100</v>
-      </c>
-      <c r="D26" t="s">
-        <v>49</v>
-      </c>
-      <c r="E26" s="1">
-        <v>45941</v>
-      </c>
-      <c r="F26" s="1">
-        <v>45945</v>
-      </c>
-      <c r="G26" t="s">
-        <v>37</v>
-      </c>
       <c r="H26" t="s">
         <v>1</v>
       </c>
       <c r="I26" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K26" s="5">
         <v>4</v>
       </c>
       <c r="L26" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="M26" t="s">
+        <v>139</v>
+      </c>
+      <c r="N26" t="s">
+        <v>2</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q26" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="R26" t="s">
+        <v>178</v>
+      </c>
+      <c r="S26" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="27" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C27" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" t="s">
+        <v>35</v>
+      </c>
+      <c r="E27" s="1">
+        <v>45925</v>
+      </c>
+      <c r="F27" s="1">
+        <v>45928</v>
+      </c>
+      <c r="G27" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" t="s">
+        <v>1</v>
+      </c>
+      <c r="I27" t="s">
+        <v>7</v>
+      </c>
+      <c r="K27" s="5">
+        <v>2</v>
+      </c>
+      <c r="L27" t="s">
+        <v>35</v>
+      </c>
+      <c r="M27" t="s">
+        <v>139</v>
+      </c>
+      <c r="N27" t="s">
+        <v>2</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P27" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q27" s="2"/>
+    </row>
+    <row r="28" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C28" t="s">
+        <v>101</v>
+      </c>
+      <c r="D28" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28" s="1">
+        <v>45933</v>
+      </c>
+      <c r="F28" s="1">
+        <v>45935</v>
+      </c>
+      <c r="G28" t="s">
+        <v>158</v>
+      </c>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q28" s="2"/>
+    </row>
+    <row r="29" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C29" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" t="s">
+        <v>48</v>
+      </c>
+      <c r="E29" s="1">
+        <v>45941</v>
+      </c>
+      <c r="F29" s="1">
+        <v>45945</v>
+      </c>
+      <c r="G29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H29" t="s">
+        <v>1</v>
+      </c>
+      <c r="I29" t="s">
+        <v>130</v>
+      </c>
+      <c r="K29" s="5">
+        <v>4</v>
+      </c>
+      <c r="L29" t="s">
+        <v>48</v>
+      </c>
+      <c r="M29" t="s">
+        <v>139</v>
+      </c>
+      <c r="N29" t="s">
+        <v>2</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P29" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>180</v>
+      </c>
+      <c r="R29" t="s">
+        <v>173</v>
+      </c>
+      <c r="S29" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="30" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C30" t="s">
+        <v>103</v>
+      </c>
+      <c r="D30" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="1">
+        <v>45986</v>
+      </c>
+      <c r="F30" s="1">
+        <v>45991</v>
+      </c>
+      <c r="G30" t="s">
+        <v>121</v>
+      </c>
+      <c r="H30" t="s">
+        <v>120</v>
+      </c>
+      <c r="I30" t="s">
+        <v>135</v>
+      </c>
+      <c r="K30" s="5">
+        <v>2</v>
+      </c>
+      <c r="L30" t="s">
+        <v>62</v>
+      </c>
+      <c r="M30" t="s">
+        <v>139</v>
+      </c>
+      <c r="N30" t="s">
+        <v>2</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P30" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q30" s="2"/>
+    </row>
+    <row r="31" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C31" t="s">
+        <v>104</v>
+      </c>
+      <c r="D31" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="1">
+        <v>45997</v>
+      </c>
+      <c r="F31" s="1">
+        <v>45997</v>
+      </c>
+      <c r="G31" t="s">
+        <v>38</v>
+      </c>
+      <c r="H31" t="s">
+        <v>1</v>
+      </c>
+      <c r="I31" t="s">
+        <v>131</v>
+      </c>
+      <c r="K31" s="5">
+        <v>2</v>
+      </c>
+      <c r="L31" t="s">
+        <v>55</v>
+      </c>
+      <c r="M31" t="s">
+        <v>140</v>
+      </c>
+      <c r="N31" t="s">
+        <v>2</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P31" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q31" s="2"/>
+    </row>
+    <row r="32" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C32" t="s">
+        <v>105</v>
+      </c>
+      <c r="D32" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" s="1">
+        <v>46004</v>
+      </c>
+      <c r="F32" s="1">
+        <v>46004</v>
+      </c>
+      <c r="G32" t="s">
+        <v>37</v>
+      </c>
+      <c r="H32" t="s">
+        <v>1</v>
+      </c>
+      <c r="I32" t="s">
+        <v>138</v>
+      </c>
+      <c r="K32" s="5">
+        <v>2</v>
+      </c>
+      <c r="L32" t="s">
+        <v>56</v>
+      </c>
+      <c r="M32" t="s">
+        <v>140</v>
+      </c>
+      <c r="N32" t="s">
+        <v>2</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q32" s="2"/>
+    </row>
+    <row r="33" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C33" t="s">
+        <v>106</v>
+      </c>
+      <c r="D33" t="s">
         <v>142</v>
       </c>
-      <c r="N26" t="s">
-        <v>2</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="27" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C27" t="s">
-        <v>101</v>
-      </c>
-      <c r="D27" t="s">
-        <v>63</v>
-      </c>
-      <c r="E27" s="1">
-        <v>45986</v>
-      </c>
-      <c r="F27" s="1">
-        <v>45991</v>
-      </c>
-      <c r="G27" t="s">
-        <v>122</v>
-      </c>
-      <c r="H27" t="s">
-        <v>121</v>
-      </c>
-      <c r="I27" t="s">
-        <v>138</v>
-      </c>
-      <c r="K27" s="5">
-        <v>2</v>
-      </c>
-      <c r="L27" t="s">
-        <v>63</v>
-      </c>
-      <c r="M27" t="s">
-        <v>142</v>
-      </c>
-      <c r="N27" t="s">
-        <v>2</v>
-      </c>
-      <c r="O27" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="2"/>
-    </row>
-    <row r="28" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C28" t="s">
-        <v>102</v>
-      </c>
-      <c r="D28" t="s">
-        <v>56</v>
-      </c>
-      <c r="E28" s="1">
-        <v>45997</v>
-      </c>
-      <c r="F28" s="1">
-        <v>45997</v>
-      </c>
-      <c r="G28" t="s">
-        <v>39</v>
-      </c>
-      <c r="H28" t="s">
-        <v>1</v>
-      </c>
-      <c r="I28" t="s">
-        <v>134</v>
-      </c>
-      <c r="K28" s="5">
-        <v>2</v>
-      </c>
-      <c r="L28" t="s">
-        <v>56</v>
-      </c>
-      <c r="M28" t="s">
-        <v>143</v>
-      </c>
-      <c r="N28" t="s">
-        <v>2</v>
-      </c>
-      <c r="O28" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="2"/>
-    </row>
-    <row r="29" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C29" t="s">
-        <v>103</v>
-      </c>
-      <c r="D29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E29" s="1">
-        <v>46004</v>
-      </c>
-      <c r="F29" s="1">
-        <v>46004</v>
-      </c>
-      <c r="G29" t="s">
-        <v>38</v>
-      </c>
-      <c r="H29" t="s">
-        <v>1</v>
-      </c>
-      <c r="I29" t="s">
-        <v>141</v>
-      </c>
-      <c r="K29" s="5">
-        <v>2</v>
-      </c>
-      <c r="L29" t="s">
-        <v>57</v>
-      </c>
-      <c r="M29" t="s">
-        <v>143</v>
-      </c>
-      <c r="N29" t="s">
-        <v>2</v>
-      </c>
-      <c r="O29" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="2"/>
-    </row>
-    <row r="30" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C30" t="s">
-        <v>104</v>
-      </c>
-      <c r="D30" t="s">
-        <v>145</v>
-      </c>
-      <c r="E30" s="1">
+      <c r="E33" s="1">
         <v>46010</v>
       </c>
-      <c r="F30" s="1">
-        <v>46010</v>
-      </c>
-      <c r="G30" t="s">
-        <v>149</v>
-      </c>
-      <c r="H30" t="s">
-        <v>1</v>
-      </c>
-      <c r="I30" t="s">
-        <v>134</v>
-      </c>
-      <c r="K30" s="5">
-        <v>4</v>
-      </c>
-      <c r="L30" t="s">
-        <v>145</v>
-      </c>
-      <c r="M30" t="s">
-        <v>142</v>
-      </c>
-      <c r="N30" t="s">
-        <v>2</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="2"/>
-    </row>
-    <row r="31" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C31" t="s">
-        <v>105</v>
-      </c>
-      <c r="D31" t="s">
-        <v>58</v>
-      </c>
-      <c r="E31" s="1">
-        <v>46019</v>
-      </c>
-      <c r="F31" s="1">
-        <v>46019</v>
-      </c>
-      <c r="G31" t="s">
-        <v>39</v>
-      </c>
-      <c r="H31" t="s">
-        <v>1</v>
-      </c>
-      <c r="I31" t="s">
-        <v>134</v>
-      </c>
-      <c r="K31" s="5">
-        <v>2</v>
-      </c>
-      <c r="L31" t="s">
-        <v>58</v>
-      </c>
-      <c r="M31" t="s">
-        <v>143</v>
-      </c>
-      <c r="N31" t="s">
-        <v>2</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="2"/>
-    </row>
-    <row r="32" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C32" t="s">
-        <v>106</v>
-      </c>
-      <c r="D32" t="s">
-        <v>59</v>
-      </c>
-      <c r="E32" s="1">
-        <v>46021</v>
-      </c>
-      <c r="F32" s="1">
-        <v>46021</v>
-      </c>
-      <c r="G32" t="s">
-        <v>21</v>
-      </c>
-      <c r="H32" t="s">
-        <v>1</v>
-      </c>
-      <c r="I32" t="s">
-        <v>134</v>
-      </c>
-      <c r="K32" s="5">
-        <v>2</v>
-      </c>
-      <c r="L32" t="s">
-        <v>59</v>
-      </c>
-      <c r="M32" t="s">
-        <v>143</v>
-      </c>
-      <c r="N32" t="s">
-        <v>2</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P32" s="1"/>
-      <c r="Q32" s="2"/>
-    </row>
-    <row r="33" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C33" t="s">
-        <v>107</v>
-      </c>
-      <c r="D33" t="s">
-        <v>61</v>
-      </c>
-      <c r="E33" s="1">
-        <v>46028</v>
-      </c>
       <c r="F33" s="1">
-        <v>46032</v>
+        <v>46012</v>
       </c>
       <c r="G33" t="s">
-        <v>40</v>
+        <v>146</v>
       </c>
       <c r="H33" t="s">
         <v>1</v>
       </c>
       <c r="I33" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="K33" s="5">
         <v>4</v>
       </c>
       <c r="L33" t="s">
-        <v>61</v>
+        <v>142</v>
       </c>
       <c r="M33" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="N33" t="s">
         <v>2</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P33" s="1"/>
-      <c r="Q33" s="2"/>
-    </row>
-    <row r="34" spans="3:17" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="P33" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q33" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="R33" t="s">
+        <v>175</v>
+      </c>
+      <c r="S33" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C34" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" t="s">
+        <v>57</v>
+      </c>
+      <c r="E34" s="1">
+        <v>46019</v>
+      </c>
+      <c r="F34" s="1">
+        <v>46019</v>
+      </c>
+      <c r="G34" t="s">
+        <v>38</v>
+      </c>
+      <c r="H34" t="s">
+        <v>1</v>
+      </c>
+      <c r="I34" t="s">
+        <v>131</v>
+      </c>
+      <c r="K34" s="5">
+        <v>2</v>
+      </c>
+      <c r="L34" t="s">
+        <v>57</v>
+      </c>
+      <c r="M34" t="s">
+        <v>140</v>
+      </c>
+      <c r="N34" t="s">
+        <v>2</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P34" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q34" s="2"/>
+    </row>
+    <row r="35" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C35" t="s">
         <v>108</v>
       </c>
-      <c r="D34" t="s">
-        <v>64</v>
-      </c>
-      <c r="E34" s="1">
-        <v>46038</v>
-      </c>
-      <c r="F34" s="1">
-        <v>46041</v>
-      </c>
-      <c r="G34" t="s">
-        <v>150</v>
-      </c>
-      <c r="H34" t="s">
-        <v>121</v>
-      </c>
-      <c r="I34" t="s">
-        <v>136</v>
-      </c>
-      <c r="K34" s="5">
-        <v>4</v>
-      </c>
-      <c r="L34" t="s">
-        <v>64</v>
-      </c>
-      <c r="M34" t="s">
-        <v>142</v>
-      </c>
-      <c r="N34" t="s">
-        <v>2</v>
-      </c>
-      <c r="O34" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P34" s="1"/>
-      <c r="Q34" s="2"/>
-    </row>
-    <row r="35" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C35" t="s">
+      <c r="D35" t="s">
+        <v>58</v>
+      </c>
+      <c r="E35" s="1">
+        <v>46021</v>
+      </c>
+      <c r="F35" s="1">
+        <v>46021</v>
+      </c>
+      <c r="G35" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" t="s">
+        <v>1</v>
+      </c>
+      <c r="I35" t="s">
+        <v>131</v>
+      </c>
+      <c r="K35" s="5">
+        <v>2</v>
+      </c>
+      <c r="L35" t="s">
+        <v>58</v>
+      </c>
+      <c r="M35" t="s">
+        <v>140</v>
+      </c>
+      <c r="N35" t="s">
+        <v>2</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P35" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q35" s="2"/>
+    </row>
+    <row r="36" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C36" t="s">
         <v>109</v>
       </c>
-      <c r="D35" t="s">
-        <v>65</v>
-      </c>
-      <c r="E35" s="1">
-        <v>46064</v>
-      </c>
-      <c r="F35" s="1">
-        <v>46069</v>
-      </c>
-      <c r="G35" t="s">
-        <v>147</v>
-      </c>
-      <c r="H35" t="s">
-        <v>1</v>
-      </c>
-      <c r="I35" t="s">
-        <v>138</v>
-      </c>
-      <c r="K35" s="5">
-        <v>5</v>
-      </c>
-      <c r="L35" t="s">
-        <v>65</v>
-      </c>
-      <c r="M35" t="s">
-        <v>142</v>
-      </c>
-      <c r="N35" t="s">
-        <v>2</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P35" s="1"/>
-      <c r="Q35" s="2"/>
-    </row>
-    <row r="36" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C36" t="s">
-        <v>110</v>
-      </c>
       <c r="D36" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E36" s="1">
-        <v>46073</v>
+        <v>46028</v>
       </c>
       <c r="F36" s="1">
-        <v>46075</v>
+        <v>46032</v>
       </c>
       <c r="G36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H36" t="s">
         <v>1</v>
@@ -2225,41 +2461,43 @@
         <v>135</v>
       </c>
       <c r="K36" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L36" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="M36" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="N36" t="s">
         <v>2</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P36" s="1"/>
+        <v>139</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="Q36" s="2"/>
     </row>
-    <row r="37" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C37" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D37" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E37" s="1">
-        <v>46109</v>
+        <v>46038</v>
       </c>
       <c r="F37" s="1">
-        <v>46118</v>
+        <v>46041</v>
       </c>
       <c r="G37" t="s">
-        <v>42</v>
+        <v>147</v>
       </c>
       <c r="H37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I37" t="s">
         <v>133</v>
@@ -2268,417 +2506,570 @@
         <v>4</v>
       </c>
       <c r="L37" t="s">
+        <v>63</v>
+      </c>
+      <c r="M37" t="s">
+        <v>139</v>
+      </c>
+      <c r="N37" t="s">
+        <v>2</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P37" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q37" s="2"/>
+    </row>
+    <row r="38" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C38" t="s">
+        <v>111</v>
+      </c>
+      <c r="D38" t="s">
+        <v>64</v>
+      </c>
+      <c r="E38" s="1">
+        <v>46064</v>
+      </c>
+      <c r="F38" s="1">
+        <v>46069</v>
+      </c>
+      <c r="G38" t="s">
+        <v>144</v>
+      </c>
+      <c r="H38" t="s">
+        <v>1</v>
+      </c>
+      <c r="I38" t="s">
+        <v>135</v>
+      </c>
+      <c r="K38" s="5">
+        <v>5</v>
+      </c>
+      <c r="L38" t="s">
+        <v>64</v>
+      </c>
+      <c r="M38" t="s">
+        <v>139</v>
+      </c>
+      <c r="N38" t="s">
+        <v>2</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P38" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q38" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="R38" t="s">
+        <v>182</v>
+      </c>
+      <c r="S38" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="39" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C39" t="s">
+        <v>112</v>
+      </c>
+      <c r="D39" t="s">
+        <v>65</v>
+      </c>
+      <c r="E39" s="1">
+        <v>46073</v>
+      </c>
+      <c r="F39" s="1">
+        <v>46075</v>
+      </c>
+      <c r="G39" t="s">
+        <v>40</v>
+      </c>
+      <c r="H39" t="s">
+        <v>1</v>
+      </c>
+      <c r="I39" t="s">
+        <v>132</v>
+      </c>
+      <c r="K39" s="5">
+        <v>2</v>
+      </c>
+      <c r="L39" t="s">
+        <v>65</v>
+      </c>
+      <c r="M39" t="s">
+        <v>140</v>
+      </c>
+      <c r="N39" t="s">
+        <v>2</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q39" s="2"/>
+    </row>
+    <row r="40" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C40" t="s">
+        <v>113</v>
+      </c>
+      <c r="D40" t="s">
+        <v>66</v>
+      </c>
+      <c r="E40" s="1">
+        <v>46109</v>
+      </c>
+      <c r="F40" s="1">
+        <v>46118</v>
+      </c>
+      <c r="G40" t="s">
+        <v>41</v>
+      </c>
+      <c r="H40" t="s">
+        <v>120</v>
+      </c>
+      <c r="I40" t="s">
+        <v>130</v>
+      </c>
+      <c r="K40" s="5">
+        <v>4</v>
+      </c>
+      <c r="L40" t="s">
+        <v>66</v>
+      </c>
+      <c r="M40" t="s">
+        <v>139</v>
+      </c>
+      <c r="N40" t="s">
+        <v>2</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P40" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q40" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="R40" t="s">
+        <v>184</v>
+      </c>
+      <c r="S40" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="41" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C41" t="s">
+        <v>114</v>
+      </c>
+      <c r="D41" t="s">
         <v>67</v>
       </c>
-      <c r="M37" t="s">
-        <v>142</v>
-      </c>
-      <c r="N37" t="s">
-        <v>2</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P37" s="1"/>
-      <c r="Q37" s="2"/>
-    </row>
-    <row r="38" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C38" t="s">
-        <v>112</v>
-      </c>
-      <c r="D38" t="s">
-        <v>68</v>
-      </c>
-      <c r="E38" s="1">
+      <c r="E41" s="1">
         <v>46123</v>
       </c>
-      <c r="F38" s="1">
+      <c r="F41" s="1">
         <v>46123</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G41" t="s">
+        <v>42</v>
+      </c>
+      <c r="H41" t="s">
+        <v>1</v>
+      </c>
+      <c r="I41" t="s">
+        <v>129</v>
+      </c>
+      <c r="K41" s="5">
+        <v>2</v>
+      </c>
+      <c r="L41" t="s">
+        <v>67</v>
+      </c>
+      <c r="M41" t="s">
+        <v>140</v>
+      </c>
+      <c r="N41" t="s">
+        <v>2</v>
+      </c>
+      <c r="O41" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P41" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q41" s="2"/>
+    </row>
+    <row r="42" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C42" t="s">
+        <v>115</v>
+      </c>
+      <c r="D42" t="s">
+        <v>70</v>
+      </c>
+      <c r="E42" s="1">
+        <v>46156</v>
+      </c>
+      <c r="F42" s="1">
+        <v>46159</v>
+      </c>
+      <c r="G42" t="s">
         <v>43</v>
       </c>
-      <c r="H38" t="s">
-        <v>1</v>
-      </c>
-      <c r="I38" t="s">
-        <v>132</v>
-      </c>
-      <c r="K38" s="5">
-        <v>2</v>
-      </c>
-      <c r="L38" t="s">
-        <v>68</v>
-      </c>
-      <c r="M38" t="s">
-        <v>143</v>
-      </c>
-      <c r="N38" t="s">
-        <v>2</v>
-      </c>
-      <c r="O38" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P38" s="1"/>
-      <c r="Q38" s="2"/>
-    </row>
-    <row r="39" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C39" t="s">
-        <v>113</v>
-      </c>
-      <c r="D39" t="s">
+      <c r="H42" t="s">
+        <v>1</v>
+      </c>
+      <c r="I42" t="s">
+        <v>133</v>
+      </c>
+      <c r="K42" s="5">
+        <v>2</v>
+      </c>
+      <c r="L42" t="s">
+        <v>70</v>
+      </c>
+      <c r="M42" t="s">
+        <v>139</v>
+      </c>
+      <c r="N42" t="s">
+        <v>2</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P42" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q42" s="2"/>
+    </row>
+    <row r="43" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C43" t="s">
+        <v>116</v>
+      </c>
+      <c r="D43" t="s">
         <v>71</v>
       </c>
-      <c r="E39" s="1">
-        <v>46156</v>
-      </c>
-      <c r="F39" s="1">
-        <v>46159</v>
-      </c>
-      <c r="G39" t="s">
+      <c r="E43" s="1">
+        <v>46165</v>
+      </c>
+      <c r="F43" s="1">
+        <v>46165</v>
+      </c>
+      <c r="G43" t="s">
+        <v>38</v>
+      </c>
+      <c r="H43" t="s">
+        <v>1</v>
+      </c>
+      <c r="I43" t="s">
+        <v>129</v>
+      </c>
+      <c r="K43" s="5">
+        <v>2</v>
+      </c>
+      <c r="L43" t="s">
+        <v>71</v>
+      </c>
+      <c r="M43" t="s">
+        <v>140</v>
+      </c>
+      <c r="N43" t="s">
+        <v>2</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q43" s="2"/>
+    </row>
+    <row r="44" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C44" t="s">
+        <v>117</v>
+      </c>
+      <c r="D44" t="s">
+        <v>72</v>
+      </c>
+      <c r="E44" s="1">
+        <v>46166</v>
+      </c>
+      <c r="F44" s="1">
+        <v>46166</v>
+      </c>
+      <c r="G44" t="s">
+        <v>20</v>
+      </c>
+      <c r="H44" t="s">
+        <v>1</v>
+      </c>
+      <c r="I44" t="s">
+        <v>136</v>
+      </c>
+      <c r="K44" s="5">
+        <v>2</v>
+      </c>
+      <c r="L44" t="s">
+        <v>72</v>
+      </c>
+      <c r="M44" t="s">
+        <v>139</v>
+      </c>
+      <c r="N44" t="s">
+        <v>2</v>
+      </c>
+      <c r="O44" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P44" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q44" s="2"/>
+    </row>
+    <row r="45" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C45" t="s">
+        <v>118</v>
+      </c>
+      <c r="D45" t="s">
+        <v>73</v>
+      </c>
+      <c r="E45" s="1">
+        <v>46177</v>
+      </c>
+      <c r="F45" s="1">
+        <v>46180</v>
+      </c>
+      <c r="G45" t="s">
         <v>44</v>
       </c>
-      <c r="H39" t="s">
-        <v>1</v>
-      </c>
-      <c r="I39" t="s">
-        <v>136</v>
-      </c>
-      <c r="K39" s="5">
-        <v>2</v>
-      </c>
-      <c r="L39" t="s">
-        <v>71</v>
-      </c>
-      <c r="M39" t="s">
-        <v>142</v>
-      </c>
-      <c r="N39" t="s">
-        <v>2</v>
-      </c>
-      <c r="O39" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P39" s="1"/>
-      <c r="Q39" s="2"/>
-    </row>
-    <row r="40" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C40" t="s">
-        <v>114</v>
-      </c>
-      <c r="D40" t="s">
-        <v>72</v>
-      </c>
-      <c r="E40" s="1">
-        <v>46165</v>
-      </c>
-      <c r="F40" s="1">
-        <v>46165</v>
-      </c>
-      <c r="G40" t="s">
-        <v>39</v>
-      </c>
-      <c r="H40" t="s">
-        <v>1</v>
-      </c>
-      <c r="I40" t="s">
-        <v>132</v>
-      </c>
-      <c r="K40" s="5">
-        <v>2</v>
-      </c>
-      <c r="L40" t="s">
-        <v>72</v>
-      </c>
-      <c r="M40" t="s">
-        <v>143</v>
-      </c>
-      <c r="N40" t="s">
-        <v>2</v>
-      </c>
-      <c r="O40" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P40" s="1"/>
-      <c r="Q40" s="2"/>
-    </row>
-    <row r="41" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C41" t="s">
-        <v>115</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="H45" t="s">
+        <v>1</v>
+      </c>
+      <c r="I45" t="s">
+        <v>133</v>
+      </c>
+      <c r="K45" s="5">
+        <v>2</v>
+      </c>
+      <c r="L45" t="s">
         <v>73</v>
       </c>
-      <c r="E41" s="1">
-        <v>46166</v>
-      </c>
-      <c r="F41" s="1">
-        <v>46166</v>
-      </c>
-      <c r="G41" t="s">
-        <v>20</v>
-      </c>
-      <c r="H41" t="s">
-        <v>1</v>
-      </c>
-      <c r="I41" t="s">
-        <v>139</v>
-      </c>
-      <c r="K41" s="5">
-        <v>2</v>
-      </c>
-      <c r="L41" t="s">
-        <v>73</v>
-      </c>
-      <c r="M41" t="s">
-        <v>142</v>
-      </c>
-      <c r="N41" t="s">
-        <v>2</v>
-      </c>
-      <c r="O41" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P41" s="1"/>
-      <c r="Q41" s="2"/>
-    </row>
-    <row r="42" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C42" t="s">
-        <v>116</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="M45" t="s">
+        <v>139</v>
+      </c>
+      <c r="N45" t="s">
+        <v>2</v>
+      </c>
+      <c r="O45" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P45" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q45" s="2"/>
+    </row>
+    <row r="46" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C46" t="s">
+        <v>119</v>
+      </c>
+      <c r="D46" t="s">
         <v>74</v>
       </c>
-      <c r="E42" s="1">
-        <v>46177</v>
-      </c>
-      <c r="F42" s="1">
-        <v>46180</v>
-      </c>
-      <c r="G42" t="s">
+      <c r="E46" s="1">
+        <v>46191</v>
+      </c>
+      <c r="F46" s="1">
+        <v>46194</v>
+      </c>
+      <c r="G46" t="s">
         <v>45</v>
       </c>
-      <c r="H42" t="s">
-        <v>1</v>
-      </c>
-      <c r="I42" t="s">
-        <v>136</v>
-      </c>
-      <c r="K42" s="5">
-        <v>2</v>
-      </c>
-      <c r="L42" t="s">
+      <c r="H46" t="s">
+        <v>1</v>
+      </c>
+      <c r="I46" t="s">
+        <v>133</v>
+      </c>
+      <c r="K46" s="5">
+        <v>2</v>
+      </c>
+      <c r="L46" t="s">
         <v>74</v>
       </c>
-      <c r="M42" t="s">
-        <v>142</v>
-      </c>
-      <c r="N42" t="s">
-        <v>2</v>
-      </c>
-      <c r="O42" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P42" s="1"/>
-      <c r="Q42" s="2"/>
-    </row>
-    <row r="43" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C43" t="s">
-        <v>117</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="M46" t="s">
+        <v>139</v>
+      </c>
+      <c r="N46" t="s">
+        <v>2</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P46" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q46" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="R46" t="s">
+        <v>186</v>
+      </c>
+      <c r="S46" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="47" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C47" t="s">
+        <v>151</v>
+      </c>
+      <c r="D47" t="s">
         <v>75</v>
       </c>
-      <c r="E43" s="1">
-        <v>46191</v>
-      </c>
-      <c r="F43" s="1">
-        <v>46194</v>
-      </c>
-      <c r="G43" t="s">
+      <c r="E47" s="1">
+        <v>46206</v>
+      </c>
+      <c r="F47" s="1">
+        <v>46215</v>
+      </c>
+      <c r="G47" t="s">
         <v>46</v>
       </c>
-      <c r="H43" t="s">
-        <v>1</v>
-      </c>
-      <c r="I43" t="s">
-        <v>136</v>
-      </c>
-      <c r="K43" s="5">
-        <v>2</v>
-      </c>
-      <c r="L43" t="s">
+      <c r="H47" t="s">
+        <v>1</v>
+      </c>
+      <c r="I47" t="s">
+        <v>130</v>
+      </c>
+      <c r="K47" s="5">
+        <v>6</v>
+      </c>
+      <c r="L47" t="s">
         <v>75</v>
       </c>
-      <c r="M43" t="s">
-        <v>142</v>
-      </c>
-      <c r="N43" t="s">
-        <v>2</v>
-      </c>
-      <c r="O43" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P43" s="1"/>
-      <c r="Q43" s="2"/>
-    </row>
-    <row r="44" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C44" t="s">
-        <v>118</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="M47" t="s">
+        <v>139</v>
+      </c>
+      <c r="N47" t="s">
+        <v>2</v>
+      </c>
+      <c r="O47" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P47" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q47" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="R47" t="s">
+        <v>188</v>
+      </c>
+      <c r="S47" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="48" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C48" t="s">
+        <v>152</v>
+      </c>
+      <c r="D48" t="s">
         <v>76</v>
       </c>
-      <c r="E44" s="1">
-        <v>46206</v>
-      </c>
-      <c r="F44" s="1">
-        <v>46215</v>
-      </c>
-      <c r="G44" t="s">
+      <c r="E48" s="1">
+        <v>46220</v>
+      </c>
+      <c r="F48" s="1">
+        <v>46222</v>
+      </c>
+      <c r="G48" t="s">
         <v>47</v>
       </c>
-      <c r="H44" t="s">
-        <v>1</v>
-      </c>
-      <c r="I44" t="s">
-        <v>133</v>
-      </c>
-      <c r="K44" s="5">
-        <v>6</v>
-      </c>
-      <c r="L44" t="s">
+      <c r="H48" t="s">
+        <v>1</v>
+      </c>
+      <c r="I48" t="s">
+        <v>135</v>
+      </c>
+      <c r="K48" s="5">
+        <v>2</v>
+      </c>
+      <c r="L48" t="s">
         <v>76</v>
       </c>
-      <c r="M44" t="s">
-        <v>142</v>
-      </c>
-      <c r="N44" t="s">
-        <v>2</v>
-      </c>
-      <c r="O44" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P44" s="1"/>
-      <c r="Q44" s="2"/>
-    </row>
-    <row r="45" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C45" t="s">
-        <v>119</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="M48" t="s">
+        <v>139</v>
+      </c>
+      <c r="N48" t="s">
+        <v>2</v>
+      </c>
+      <c r="O48" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P48" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q48" s="2"/>
+    </row>
+    <row r="49" spans="3:17" x14ac:dyDescent="0.2">
+      <c r="C49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D49" t="s">
         <v>77</v>
       </c>
-      <c r="E45" s="1">
-        <v>46220</v>
-      </c>
-      <c r="F45" s="1">
-        <v>46222</v>
-      </c>
-      <c r="G45" t="s">
-        <v>48</v>
-      </c>
-      <c r="H45" t="s">
-        <v>1</v>
-      </c>
-      <c r="I45" t="s">
-        <v>138</v>
-      </c>
-      <c r="K45" s="5">
-        <v>2</v>
-      </c>
-      <c r="L45" t="s">
+      <c r="E49" s="1">
+        <v>46234</v>
+      </c>
+      <c r="F49" s="1">
+        <v>46236</v>
+      </c>
+      <c r="G49" t="s">
+        <v>78</v>
+      </c>
+      <c r="H49" t="s">
+        <v>1</v>
+      </c>
+      <c r="I49" t="s">
+        <v>134</v>
+      </c>
+      <c r="K49" s="5">
+        <v>4</v>
+      </c>
+      <c r="L49" t="s">
         <v>77</v>
       </c>
-      <c r="M45" t="s">
-        <v>142</v>
-      </c>
-      <c r="N45" t="s">
-        <v>2</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P45" s="1"/>
-      <c r="Q45" s="2"/>
-    </row>
-    <row r="46" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C46" t="s">
-        <v>120</v>
-      </c>
-      <c r="D46" t="s">
-        <v>78</v>
-      </c>
-      <c r="E46" s="1">
-        <v>46234</v>
-      </c>
-      <c r="F46" s="1">
-        <v>46236</v>
-      </c>
-      <c r="G46" t="s">
-        <v>79</v>
-      </c>
-      <c r="H46" t="s">
-        <v>1</v>
-      </c>
-      <c r="I46" t="s">
-        <v>137</v>
-      </c>
-      <c r="K46" s="5">
-        <v>4</v>
-      </c>
-      <c r="L46" t="s">
-        <v>78</v>
-      </c>
-      <c r="M46" t="s">
-        <v>142</v>
-      </c>
-      <c r="N46" t="s">
-        <v>2</v>
-      </c>
-      <c r="O46" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="P46" s="1"/>
-      <c r="Q46" s="2"/>
-    </row>
-    <row r="47" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="P47" s="1"/>
-      <c r="Q47" s="2"/>
-    </row>
-    <row r="48" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="C48" t="s">
+      <c r="M49" t="s">
+        <v>139</v>
+      </c>
+      <c r="N49" t="s">
+        <v>2</v>
+      </c>
+      <c r="O49" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="P49" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q49" s="2"/>
+    </row>
+    <row r="50" spans="3:17" x14ac:dyDescent="0.2">
+      <c r="P50" s="1"/>
+      <c r="Q50" s="2"/>
+    </row>
+    <row r="51" spans="3:17" x14ac:dyDescent="0.2">
+      <c r="C51" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C49" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C50" t="s">
+    <row r="54" spans="3:17" x14ac:dyDescent="0.2">
+      <c r="C54" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C51" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C52" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C53" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C54" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version 0.9 - Add privacy-safe public build pipeline
</commit_message>
<xml_diff>
--- a/travelogue/data/Travelogue Data.xlsx
+++ b/travelogue/data/Travelogue Data.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gscott/Travelogue/travelogue/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AEF414-757C-9944-8334-1E6C6B8A45BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A097A26-C52F-8B42-9F09-57D8CFC541BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="1920" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
+    <workbookView xWindow="0" yWindow="1900" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_MailAutoSig" localSheetId="0">'Sheet1 (2)'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1 (2)'!$C$2:$J$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1 (2)'!$C$2:$K$40</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="231">
   <si>
     <t>Train</t>
   </si>
@@ -455,9 +455,6 @@
     <t>Festival</t>
   </si>
   <si>
-    <t>Volksfest</t>
-  </si>
-  <si>
     <t>Groceries</t>
   </si>
   <si>
@@ -530,27 +527,12 @@
     <t>Even in the cold of January, Paris warms our hearts.</t>
   </si>
   <si>
-    <t>The reason why George moved the family!</t>
-  </si>
-  <si>
-    <t>Refreshing swimming, delicious food, unbeatable views</t>
-  </si>
-  <si>
-    <t>Revisiting our favorite honeymoon spot almost 10 years later</t>
-  </si>
-  <si>
-    <t>Walruses for neighbors and 24-hour access to an incredible zoon</t>
-  </si>
-  <si>
     <t>First Tour de France</t>
   </si>
   <si>
     <t>First Real Trip</t>
   </si>
   <si>
-    <t>George's Favorite Birthday</t>
-  </si>
-  <si>
     <t>Favorite Ski Trip</t>
   </si>
   <si>
@@ -563,24 +545,9 @@
     <t>Big Summer Trip</t>
   </si>
   <si>
-    <t>Bucket List Country!</t>
-  </si>
-  <si>
-    <t>Christmas Market Trip</t>
-  </si>
-  <si>
-    <t>Featuring a torch-lit walk</t>
-  </si>
-  <si>
-    <t>And a 10th wedding anniversary!</t>
-  </si>
-  <si>
     <t>Fanciest Livestock</t>
   </si>
   <si>
-    <t>Cows with Hats!</t>
-  </si>
-  <si>
     <t>Most Nostalgic</t>
   </si>
   <si>
@@ -590,15 +557,9 @@
     <t>Most Awe-Inspiring</t>
   </si>
   <si>
-    <t>Being citizens of the world</t>
-  </si>
-  <si>
     <t>Best Hidden Gems</t>
   </si>
   <si>
-    <t>Get there before the influencers do!</t>
-  </si>
-  <si>
     <t>Most Provincial</t>
   </si>
   <si>
@@ -608,9 +569,6 @@
     <t>Best Mountains</t>
   </si>
   <si>
-    <t>Great hikes, food, and views</t>
-  </si>
-  <si>
     <t>IMG_0562.jpeg</t>
   </si>
   <si>
@@ -654,6 +612,129 @@
   </si>
   <si>
     <t>IMG_9794.jpeg</t>
+  </si>
+  <si>
+    <t>Public Trip Title</t>
+  </si>
+  <si>
+    <t>Volksfest with Friends</t>
+  </si>
+  <si>
+    <t>Grocery Trip</t>
+  </si>
+  <si>
+    <t>2024 Fall Trip to Austrian Alps</t>
+  </si>
+  <si>
+    <t>Weekend in Paris</t>
+  </si>
+  <si>
+    <t>2025 Ski Trip with Friends</t>
+  </si>
+  <si>
+    <t>Beach, Tulips, and Bruges</t>
+  </si>
+  <si>
+    <t>Meeting Friends in Strasbourg</t>
+  </si>
+  <si>
+    <t>Anniversary at Tour de France</t>
+  </si>
+  <si>
+    <t>September in Paris</t>
+  </si>
+  <si>
+    <t>Fall in Slovenia</t>
+  </si>
+  <si>
+    <t>Thanksgiving with Friends</t>
+  </si>
+  <si>
+    <t>Luxembourg Christmas Market with Friends</t>
+  </si>
+  <si>
+    <t>Ravenna Gorge Christmas Market</t>
+  </si>
+  <si>
+    <t>Luxembourg Christmas Market with Family</t>
+  </si>
+  <si>
+    <t>Metz Christmas Market with Family</t>
+  </si>
+  <si>
+    <t>Zurich in January</t>
+  </si>
+  <si>
+    <t>Sunny Weekend in Valencia</t>
+  </si>
+  <si>
+    <t>Sunny Weekend in Porto</t>
+  </si>
+  <si>
+    <t>French Ski Weekend</t>
+  </si>
+  <si>
+    <t>Easter in the Baltics</t>
+  </si>
+  <si>
+    <t>Luxembourg with Friends</t>
+  </si>
+  <si>
+    <t>Wissembourg Festival with Friends</t>
+  </si>
+  <si>
+    <t>Vosges Lake Weekend with Friends</t>
+  </si>
+  <si>
+    <t>Dolomites with Friends</t>
+  </si>
+  <si>
+    <t>Tour de France and Strasbourg</t>
+  </si>
+  <si>
+    <t>A Favorite Birthday</t>
+  </si>
+  <si>
+    <t>Best Christmas Market Trip</t>
+  </si>
+  <si>
+    <t>A big reason why we moved to Europe!</t>
+  </si>
+  <si>
+    <t>And a big wedding anniversary!</t>
+  </si>
+  <si>
+    <t>Refreshing swimming, delicious food, unbeatable views.</t>
+  </si>
+  <si>
+    <t>Revisiting our favorite honeymoon spot.</t>
+  </si>
+  <si>
+    <t>Walruses for neighbors and 24-hour access to an incredible zoo.</t>
+  </si>
+  <si>
+    <t>Visiting a bucket list country!</t>
+  </si>
+  <si>
+    <t>Cows with hats!</t>
+  </si>
+  <si>
+    <t>Another bucket list country!</t>
+  </si>
+  <si>
+    <t>Featuring a torch-lit walk in the Black Forest.</t>
+  </si>
+  <si>
+    <t>Love being citizens of the world.</t>
+  </si>
+  <si>
+    <t>Three wonderful countries so easy to access.</t>
+  </si>
+  <si>
+    <t>Great hikes, food, and views.</t>
+  </si>
+  <si>
+    <t>Playmobil Fun Park with Cousins</t>
   </si>
 </sst>
 </file>
@@ -749,14 +830,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:S49" totalsRowShown="0">
-  <autoFilter ref="C6:S49" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C7:S49">
-    <sortCondition ref="C6:C49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:T49" totalsRowShown="0">
+  <autoFilter ref="C6:T49" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C7:T49">
+    <sortCondition ref="F6:F49"/>
   </sortState>
-  <tableColumns count="17">
+  <tableColumns count="18">
     <tableColumn id="16" xr3:uid="{B7B8133A-8A6E-4EA5-B294-9E2634108185}" name="Trip ID"/>
     <tableColumn id="1" xr3:uid="{21A3BC19-512C-634F-86B1-18BDC46CFC75}" name="Trip Title"/>
+    <tableColumn id="18" xr3:uid="{674D4376-E77D-8B47-AAE3-937EFD02E039}" name="Public Trip Title"/>
     <tableColumn id="2" xr3:uid="{BBBE16A1-D09A-4AE1-8F63-8AFDBF217A9F}" name="Start Date" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{E56FF79B-67A8-4495-BE75-8ABC52E5DC1B}" name="End Date" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{085DA54F-08D7-43B8-B0F4-A47955988CBE}" name="Stops"/>
@@ -1097,28 +1179,29 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="C2:S54"/>
+  <dimension ref="C2:T54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="11.5" customWidth="1"/>
     <col min="4" max="4" width="48.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="79.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.1640625" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="24" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" style="5" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="48.1640625" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="0" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="10" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="9.33203125" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.1640625" customWidth="1"/>
+    <col min="6" max="6" width="11.5" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="79.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.1640625" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" style="5" customWidth="1"/>
+    <col min="13" max="13" width="48.1640625" customWidth="1"/>
+    <col min="14" max="14" width="8.83203125" customWidth="1"/>
+    <col min="15" max="15" width="10" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" customWidth="1"/>
+    <col min="17" max="17" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="31.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="49.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:19" ht="27" x14ac:dyDescent="0.35">
+    <row r="2" spans="3:20" ht="27" x14ac:dyDescent="0.35">
       <c r="C2" s="6" t="s">
         <v>9</v>
       </c>
@@ -1128,18 +1211,19 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
-    </row>
-    <row r="3" spans="3:19" x14ac:dyDescent="0.2">
-      <c r="G3" s="4"/>
-      <c r="H3" s="3"/>
-      <c r="L3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="P3" s="2"/>
-    </row>
-    <row r="4" spans="3:19" x14ac:dyDescent="0.2">
-      <c r="L4" s="2"/>
-    </row>
-    <row r="6" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="J2" s="6"/>
+    </row>
+    <row r="3" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="H3" s="4"/>
+      <c r="I3" s="3"/>
+      <c r="M3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="Q3" s="2"/>
+    </row>
+    <row r="4" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="M4" s="2"/>
+    </row>
+    <row r="6" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>79</v>
       </c>
@@ -1147,1934 +1231,2126 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
+        <v>190</v>
+      </c>
+      <c r="F6" t="s">
         <v>5</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>4</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>19</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>6</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>18</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>122</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="L6" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>124</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>125</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>8</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>126</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
+        <v>147</v>
+      </c>
+      <c r="R6" t="s">
         <v>148</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="S6" t="s">
+        <v>158</v>
+      </c>
+      <c r="T6" t="s">
         <v>149</v>
       </c>
-      <c r="R6" t="s">
-        <v>159</v>
-      </c>
-      <c r="S6" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" spans="3:19" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>80</v>
       </c>
       <c r="D7" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="1">
-        <v>45535</v>
+      <c r="E7" t="s">
+        <v>68</v>
       </c>
       <c r="F7" s="1">
         <v>45535</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="1">
+        <v>45535</v>
+      </c>
+      <c r="H7" t="s">
         <v>20</v>
       </c>
-      <c r="H7" t="s">
-        <v>1</v>
-      </c>
       <c r="I7" t="s">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
         <v>134</v>
       </c>
-      <c r="K7" s="5">
-        <v>2</v>
-      </c>
-      <c r="L7" t="s">
+      <c r="L7" s="5">
+        <v>2</v>
+      </c>
+      <c r="M7" t="s">
         <v>68</v>
       </c>
-      <c r="M7" t="s">
-        <v>139</v>
-      </c>
-      <c r="N7" t="s">
-        <v>2</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>139</v>
+      <c r="N7" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O7" t="s">
+        <v>2</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q7" s="2"/>
-    </row>
-    <row r="8" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R7" s="2"/>
+    </row>
+    <row r="8" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
         <v>81</v>
       </c>
       <c r="D8" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="1">
-        <v>45556</v>
+      <c r="E8" t="s">
+        <v>69</v>
       </c>
       <c r="F8" s="1">
         <v>45556</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="1">
+        <v>45556</v>
+      </c>
+      <c r="H8" t="s">
         <v>38</v>
       </c>
-      <c r="H8" t="s">
-        <v>1</v>
-      </c>
       <c r="I8" t="s">
+        <v>1</v>
+      </c>
+      <c r="J8" t="s">
         <v>134</v>
       </c>
-      <c r="K8" s="5">
-        <v>2</v>
-      </c>
-      <c r="L8" t="s">
+      <c r="L8" s="5">
+        <v>2</v>
+      </c>
+      <c r="M8" t="s">
         <v>69</v>
       </c>
-      <c r="M8" t="s">
-        <v>139</v>
-      </c>
-      <c r="N8" t="s">
-        <v>2</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>139</v>
+      <c r="N8" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O8" t="s">
+        <v>2</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q8" s="2"/>
-    </row>
-    <row r="9" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R8" s="2"/>
+    </row>
+    <row r="9" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C9" t="s">
         <v>82</v>
       </c>
       <c r="D9" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" t="s">
+        <v>193</v>
+      </c>
+      <c r="F9" s="1">
         <v>45592</v>
       </c>
-      <c r="F9" s="1">
+      <c r="G9" s="1">
         <v>45595</v>
       </c>
-      <c r="G9" t="s">
-        <v>141</v>
-      </c>
       <c r="H9" t="s">
-        <v>1</v>
+        <v>140</v>
       </c>
       <c r="I9" t="s">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
         <v>130</v>
       </c>
-      <c r="K9" s="5">
+      <c r="L9" s="5">
         <v>6</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>49</v>
       </c>
-      <c r="M9" t="s">
-        <v>139</v>
-      </c>
-      <c r="N9" t="s">
-        <v>2</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>139</v>
+      <c r="N9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O9" t="s">
+        <v>2</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="R9" t="s">
-        <v>160</v>
+        <v>138</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>162</v>
       </c>
       <c r="S9" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="10" spans="3:19" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+      <c r="T9" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="10" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C10" t="s">
         <v>83</v>
       </c>
       <c r="D10" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="1">
-        <v>45640</v>
+      <c r="E10" t="s">
+        <v>50</v>
       </c>
       <c r="F10" s="1">
         <v>45640</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="1">
+        <v>45640</v>
+      </c>
+      <c r="H10" t="s">
         <v>20</v>
       </c>
-      <c r="H10" t="s">
-        <v>1</v>
-      </c>
       <c r="I10" t="s">
+        <v>1</v>
+      </c>
+      <c r="J10" t="s">
         <v>131</v>
       </c>
-      <c r="K10" s="5">
-        <v>2</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="L10" s="5">
+        <v>2</v>
+      </c>
+      <c r="M10" t="s">
         <v>50</v>
       </c>
-      <c r="M10" t="s">
-        <v>139</v>
-      </c>
-      <c r="N10" t="s">
-        <v>2</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>139</v>
+      <c r="N10" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O10" t="s">
+        <v>2</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q10" s="2"/>
-    </row>
-    <row r="11" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R10" s="2"/>
+    </row>
+    <row r="11" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
         <v>84</v>
       </c>
       <c r="D11" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="1">
-        <v>45654</v>
+      <c r="E11" t="s">
+        <v>51</v>
       </c>
       <c r="F11" s="1">
         <v>45654</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="1">
+        <v>45654</v>
+      </c>
+      <c r="H11" t="s">
         <v>21</v>
       </c>
-      <c r="H11" t="s">
-        <v>1</v>
-      </c>
       <c r="I11" t="s">
+        <v>1</v>
+      </c>
+      <c r="J11" t="s">
         <v>131</v>
       </c>
-      <c r="K11" s="5">
-        <v>2</v>
-      </c>
-      <c r="L11" t="s">
+      <c r="L11" s="5">
+        <v>2</v>
+      </c>
+      <c r="M11" t="s">
         <v>51</v>
       </c>
-      <c r="M11" t="s">
-        <v>140</v>
-      </c>
       <c r="N11" t="s">
-        <v>2</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>139</v>
+        <v>139</v>
+      </c>
+      <c r="O11" t="s">
+        <v>2</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q11" s="2"/>
-    </row>
-    <row r="12" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R11" s="2"/>
+    </row>
+    <row r="12" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
         <v>85</v>
       </c>
       <c r="D12" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" t="s">
+        <v>194</v>
+      </c>
+      <c r="F12" s="1">
         <v>45667</v>
       </c>
-      <c r="F12" s="1">
+      <c r="G12" s="1">
         <v>45669</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>22</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>0</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>135</v>
       </c>
-      <c r="K12" s="5">
-        <v>2</v>
-      </c>
-      <c r="L12" t="s">
+      <c r="L12" s="5">
+        <v>2</v>
+      </c>
+      <c r="M12" t="s">
         <v>59</v>
       </c>
-      <c r="M12" t="s">
-        <v>139</v>
-      </c>
-      <c r="N12" t="s">
-        <v>2</v>
-      </c>
-      <c r="O12" s="1" t="s">
-        <v>139</v>
+      <c r="N12" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O12" t="s">
+        <v>2</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q12" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="R12" t="s">
-        <v>161</v>
+        <v>138</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="S12" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="13" spans="3:19" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+      <c r="T12" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C13" t="s">
         <v>86</v>
       </c>
       <c r="D13" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" t="s">
+        <v>207</v>
+      </c>
+      <c r="F13" s="1">
         <v>45674</v>
       </c>
-      <c r="F13" s="1">
+      <c r="G13" s="1">
         <v>45677</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>23</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>133</v>
       </c>
-      <c r="K13" s="5">
-        <v>2</v>
-      </c>
-      <c r="L13" t="s">
+      <c r="L13" s="5">
+        <v>2</v>
+      </c>
+      <c r="M13" t="s">
         <v>52</v>
       </c>
-      <c r="M13" t="s">
-        <v>139</v>
-      </c>
-      <c r="N13" t="s">
-        <v>2</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>139</v>
+      <c r="N13" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O13" t="s">
+        <v>2</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q13" s="2"/>
-    </row>
-    <row r="14" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R13" s="2"/>
+    </row>
+    <row r="14" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C14" t="s">
         <v>87</v>
       </c>
       <c r="D14" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="1">
-        <v>45705</v>
+      <c r="E14" t="s">
+        <v>53</v>
       </c>
       <c r="F14" s="1">
         <v>45705</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="1">
+        <v>45705</v>
+      </c>
+      <c r="H14" t="s">
         <v>127</v>
       </c>
-      <c r="H14" t="s">
-        <v>1</v>
-      </c>
       <c r="I14" t="s">
+        <v>1</v>
+      </c>
+      <c r="J14" t="s">
         <v>132</v>
       </c>
-      <c r="K14" s="5">
-        <v>2</v>
-      </c>
-      <c r="L14" t="s">
+      <c r="L14" s="5">
+        <v>2</v>
+      </c>
+      <c r="M14" t="s">
         <v>53</v>
       </c>
-      <c r="M14" t="s">
-        <v>139</v>
-      </c>
-      <c r="N14" t="s">
-        <v>2</v>
-      </c>
-      <c r="O14" s="1" t="s">
-        <v>139</v>
+      <c r="N14" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O14" t="s">
+        <v>2</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q14" s="2"/>
-    </row>
-    <row r="15" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R14" s="2"/>
+    </row>
+    <row r="15" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C15" t="s">
         <v>88</v>
       </c>
       <c r="D15" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" t="s">
+        <v>195</v>
+      </c>
+      <c r="F15" s="1">
         <v>45711</v>
       </c>
-      <c r="F15" s="1">
+      <c r="G15" s="1">
         <v>45718</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>25</v>
       </c>
-      <c r="H15" t="s">
-        <v>1</v>
-      </c>
       <c r="I15" t="s">
+        <v>1</v>
+      </c>
+      <c r="J15" t="s">
         <v>132</v>
       </c>
-      <c r="K15" s="5">
+      <c r="L15" s="5">
         <v>4</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>61</v>
       </c>
-      <c r="M15" t="s">
-        <v>139</v>
-      </c>
-      <c r="N15" t="s">
-        <v>2</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>139</v>
+      <c r="N15" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O15" t="s">
+        <v>2</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q15" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="R15" t="s">
-        <v>162</v>
+        <v>138</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="S15" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="16" spans="3:19" x14ac:dyDescent="0.2">
+        <v>218</v>
+      </c>
+      <c r="T15" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="16" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C16" t="s">
         <v>89</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" t="s">
+        <v>196</v>
+      </c>
+      <c r="F16" s="1">
         <v>45765</v>
       </c>
-      <c r="F16" s="1">
+      <c r="G16" s="1">
         <v>45768</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>28</v>
       </c>
-      <c r="H16" t="s">
-        <v>1</v>
-      </c>
       <c r="I16" t="s">
+        <v>1</v>
+      </c>
+      <c r="J16" t="s">
         <v>130</v>
       </c>
-      <c r="K16" s="5">
+      <c r="L16" s="5">
         <v>3</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>11</v>
       </c>
-      <c r="M16" t="s">
-        <v>139</v>
-      </c>
-      <c r="N16" t="s">
-        <v>2</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>139</v>
+      <c r="N16" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O16" t="s">
+        <v>2</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q16" s="2"/>
-    </row>
-    <row r="17" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R16" s="2"/>
+    </row>
+    <row r="17" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
         <v>90</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="1">
-        <v>45787</v>
+      <c r="E17" t="s">
+        <v>197</v>
       </c>
       <c r="F17" s="1">
         <v>45787</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="1">
+        <v>45787</v>
+      </c>
+      <c r="H17" t="s">
         <v>24</v>
       </c>
-      <c r="H17" t="s">
-        <v>1</v>
-      </c>
       <c r="I17" t="s">
+        <v>1</v>
+      </c>
+      <c r="J17" t="s">
         <v>129</v>
       </c>
-      <c r="K17" s="5">
-        <v>2</v>
-      </c>
-      <c r="L17" t="s">
+      <c r="L17" s="5">
+        <v>2</v>
+      </c>
+      <c r="M17" t="s">
         <v>12</v>
       </c>
-      <c r="M17" t="s">
-        <v>139</v>
-      </c>
-      <c r="N17" t="s">
-        <v>2</v>
-      </c>
-      <c r="O17" s="1" t="s">
-        <v>139</v>
+      <c r="N17" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O17" t="s">
+        <v>2</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q17" s="2"/>
-    </row>
-    <row r="18" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R17" s="2"/>
+    </row>
+    <row r="18" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C18" t="s">
         <v>91</v>
       </c>
       <c r="D18" t="s">
         <v>13</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="1">
         <v>45805</v>
       </c>
-      <c r="F18" s="1">
+      <c r="G18" s="1">
         <v>45809</v>
       </c>
-      <c r="G18" t="s">
-        <v>143</v>
-      </c>
       <c r="H18" t="s">
-        <v>1</v>
+        <v>142</v>
       </c>
       <c r="I18" t="s">
+        <v>1</v>
+      </c>
+      <c r="J18" t="s">
         <v>133</v>
       </c>
-      <c r="K18" s="5">
+      <c r="L18" s="5">
         <v>7</v>
       </c>
-      <c r="L18" t="s">
+      <c r="M18" t="s">
         <v>13</v>
       </c>
-      <c r="M18" t="s">
-        <v>139</v>
-      </c>
-      <c r="N18" t="s">
-        <v>2</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>139</v>
+      <c r="N18" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O18" t="s">
+        <v>2</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q18" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="R18" t="s">
-        <v>163</v>
+        <v>138</v>
+      </c>
+      <c r="Q18" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>164</v>
       </c>
       <c r="S18" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="19" spans="3:19" x14ac:dyDescent="0.2">
+        <v>220</v>
+      </c>
+      <c r="T18" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C19" t="s">
         <v>92</v>
       </c>
       <c r="D19" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" s="1">
         <v>45814</v>
       </c>
-      <c r="F19" s="1">
+      <c r="G19" s="1">
         <v>45817</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>29</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>3</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>135</v>
       </c>
-      <c r="K19" s="5">
-        <v>2</v>
-      </c>
-      <c r="L19" t="s">
+      <c r="L19" s="5">
+        <v>2</v>
+      </c>
+      <c r="M19" t="s">
         <v>54</v>
       </c>
-      <c r="M19" t="s">
-        <v>139</v>
-      </c>
-      <c r="N19" t="s">
-        <v>2</v>
-      </c>
-      <c r="O19" s="1" t="s">
-        <v>139</v>
+      <c r="N19" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O19" t="s">
+        <v>2</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q19" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R19" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="S19" t="s">
+        <v>221</v>
+      </c>
+      <c r="T19" t="s">
         <v>179</v>
       </c>
-      <c r="R19" t="s">
-        <v>164</v>
-      </c>
-      <c r="S19" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="20" spans="3:19" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C20" t="s">
         <v>93</v>
       </c>
       <c r="D20" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="1">
         <v>45842</v>
       </c>
-      <c r="F20" s="1">
+      <c r="G20" s="1">
         <v>45844</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>128</v>
       </c>
-      <c r="H20" t="s">
-        <v>1</v>
-      </c>
       <c r="I20" t="s">
+        <v>1</v>
+      </c>
+      <c r="J20" t="s">
         <v>133</v>
       </c>
-      <c r="K20" s="5">
+      <c r="L20" s="5">
         <v>4</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>14</v>
       </c>
-      <c r="M20" t="s">
-        <v>139</v>
-      </c>
-      <c r="N20" t="s">
-        <v>2</v>
-      </c>
-      <c r="O20" s="1" t="s">
-        <v>139</v>
+      <c r="N20" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O20" t="s">
+        <v>2</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q20" s="2"/>
-    </row>
-    <row r="21" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R20" s="2"/>
+    </row>
+    <row r="21" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C21" t="s">
         <v>94</v>
       </c>
       <c r="D21" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="1">
         <v>45856</v>
       </c>
-      <c r="F21" s="1">
+      <c r="G21" s="1">
         <v>45857</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>30</v>
       </c>
-      <c r="H21" t="s">
-        <v>1</v>
-      </c>
       <c r="I21" t="s">
+        <v>1</v>
+      </c>
+      <c r="J21" t="s">
         <v>134</v>
       </c>
-      <c r="K21" s="5">
+      <c r="L21" s="5">
         <v>4</v>
       </c>
-      <c r="L21" t="s">
+      <c r="M21" t="s">
         <v>15</v>
       </c>
-      <c r="M21" t="s">
-        <v>139</v>
-      </c>
-      <c r="N21" t="s">
-        <v>2</v>
-      </c>
-      <c r="O21" s="1" t="s">
-        <v>139</v>
+      <c r="N21" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O21" t="s">
+        <v>2</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q21" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="R21" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q21" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R21" s="2" t="s">
         <v>165</v>
       </c>
       <c r="S21" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="22" spans="3:19" x14ac:dyDescent="0.2">
+        <v>222</v>
+      </c>
+      <c r="T21" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="22" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C22" t="s">
         <v>95</v>
       </c>
       <c r="D22" t="s">
         <v>16</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" t="s">
+        <v>198</v>
+      </c>
+      <c r="F22" s="1">
         <v>45862</v>
       </c>
-      <c r="F22" s="1">
+      <c r="G22" s="1">
         <v>45865</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>31</v>
       </c>
-      <c r="H22" t="s">
-        <v>1</v>
-      </c>
       <c r="I22" t="s">
+        <v>1</v>
+      </c>
+      <c r="J22" t="s">
         <v>135</v>
       </c>
-      <c r="K22" s="5">
+      <c r="L22" s="5">
         <v>6</v>
       </c>
-      <c r="L22" t="s">
+      <c r="M22" t="s">
         <v>16</v>
       </c>
-      <c r="M22" t="s">
-        <v>139</v>
-      </c>
-      <c r="N22" t="s">
-        <v>2</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>139</v>
+      <c r="N22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O22" t="s">
+        <v>2</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q22" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="R22" t="s">
-        <v>176</v>
+        <v>138</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>161</v>
       </c>
       <c r="S22" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="23" spans="3:19" x14ac:dyDescent="0.2">
+        <v>219</v>
+      </c>
+      <c r="T22" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="23" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C23" t="s">
         <v>96</v>
       </c>
       <c r="D23" t="s">
-        <v>157</v>
-      </c>
-      <c r="E23" s="1">
+        <v>156</v>
+      </c>
+      <c r="E23" t="s">
+        <v>156</v>
+      </c>
+      <c r="F23" s="1">
         <v>45870</v>
       </c>
-      <c r="F23" s="1">
+      <c r="G23" s="1">
         <v>45872</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
+        <v>155</v>
+      </c>
+      <c r="I23" t="s">
+        <v>1</v>
+      </c>
+      <c r="J23" t="s">
+        <v>7</v>
+      </c>
+      <c r="L23" s="5">
+        <v>0</v>
+      </c>
+      <c r="M23" t="s">
         <v>156</v>
       </c>
-      <c r="O23" s="1"/>
+      <c r="N23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O23" t="s">
+        <v>2</v>
+      </c>
       <c r="P23" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q23" s="2"/>
-    </row>
-    <row r="24" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R23" s="2"/>
+    </row>
+    <row r="24" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C24" t="s">
         <v>97</v>
       </c>
       <c r="D24" t="s">
-        <v>155</v>
-      </c>
-      <c r="E24" s="1">
+        <v>154</v>
+      </c>
+      <c r="E24" t="s">
+        <v>154</v>
+      </c>
+      <c r="F24" s="1">
         <v>45877</v>
       </c>
-      <c r="F24" s="1">
+      <c r="G24" s="1">
         <v>45879</v>
       </c>
-      <c r="G24" t="s">
-        <v>154</v>
-      </c>
-      <c r="O24" s="1"/>
+      <c r="H24" t="s">
+        <v>153</v>
+      </c>
+      <c r="I24" t="s">
+        <v>1</v>
+      </c>
+      <c r="J24" t="s">
+        <v>134</v>
+      </c>
+      <c r="L24" s="5">
+        <v>0</v>
+      </c>
+      <c r="M24" t="s">
+        <v>230</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O24" t="s">
+        <v>2</v>
+      </c>
       <c r="P24" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q24" s="2"/>
-    </row>
-    <row r="25" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R24" s="2"/>
+    </row>
+    <row r="25" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C25" t="s">
         <v>98</v>
       </c>
       <c r="D25" t="s">
         <v>17</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="1">
         <v>45885</v>
       </c>
-      <c r="F25" s="1">
+      <c r="G25" s="1">
         <v>45890</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>32</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>120</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>130</v>
       </c>
-      <c r="K25" s="5">
-        <v>2</v>
-      </c>
-      <c r="L25" t="s">
+      <c r="L25" s="5">
+        <v>2</v>
+      </c>
+      <c r="M25" t="s">
         <v>17</v>
       </c>
-      <c r="M25" t="s">
-        <v>139</v>
-      </c>
-      <c r="N25" t="s">
-        <v>2</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>139</v>
+      <c r="N25" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O25" t="s">
+        <v>2</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q25" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="R25" t="s">
-        <v>173</v>
+        <v>138</v>
+      </c>
+      <c r="Q25" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R25" s="2" t="s">
+        <v>166</v>
       </c>
       <c r="S25" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="26" spans="3:19" x14ac:dyDescent="0.2">
+        <v>223</v>
+      </c>
+      <c r="T25" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C26" t="s">
         <v>99</v>
       </c>
       <c r="D26" t="s">
-        <v>145</v>
-      </c>
-      <c r="E26" s="1">
+        <v>144</v>
+      </c>
+      <c r="E26" t="s">
+        <v>144</v>
+      </c>
+      <c r="F26" s="1">
         <v>45905</v>
       </c>
-      <c r="F26" s="1">
+      <c r="G26" s="1">
         <v>45907</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>33</v>
       </c>
-      <c r="H26" t="s">
-        <v>1</v>
-      </c>
       <c r="I26" t="s">
+        <v>1</v>
+      </c>
+      <c r="J26" t="s">
         <v>136</v>
       </c>
-      <c r="K26" s="5">
+      <c r="L26" s="5">
         <v>4</v>
       </c>
-      <c r="L26" t="s">
+      <c r="M26" t="s">
         <v>34</v>
       </c>
-      <c r="M26" t="s">
-        <v>139</v>
-      </c>
-      <c r="N26" t="s">
-        <v>2</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>139</v>
+      <c r="N26" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O26" t="s">
+        <v>2</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q26" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="R26" t="s">
-        <v>178</v>
+        <v>138</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R26" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="S26" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="27" spans="3:19" x14ac:dyDescent="0.2">
+        <v>224</v>
+      </c>
+      <c r="T26" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="27" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C27" t="s">
         <v>100</v>
       </c>
       <c r="D27" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" s="1">
         <v>45925</v>
       </c>
-      <c r="F27" s="1">
+      <c r="G27" s="1">
         <v>45928</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>22</v>
       </c>
-      <c r="H27" t="s">
-        <v>1</v>
-      </c>
       <c r="I27" t="s">
+        <v>1</v>
+      </c>
+      <c r="J27" t="s">
         <v>7</v>
       </c>
-      <c r="K27" s="5">
-        <v>2</v>
-      </c>
-      <c r="L27" t="s">
+      <c r="L27" s="5">
+        <v>2</v>
+      </c>
+      <c r="M27" t="s">
         <v>35</v>
       </c>
-      <c r="M27" t="s">
-        <v>139</v>
-      </c>
-      <c r="N27" t="s">
-        <v>2</v>
-      </c>
-      <c r="O27" s="1" t="s">
-        <v>139</v>
+      <c r="N27" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O27" t="s">
+        <v>2</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q27" s="2"/>
-    </row>
-    <row r="28" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q27" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R27" s="2"/>
+    </row>
+    <row r="28" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C28" t="s">
         <v>101</v>
       </c>
       <c r="D28" t="s">
-        <v>137</v>
-      </c>
-      <c r="E28" s="1">
+        <v>191</v>
+      </c>
+      <c r="E28" t="s">
+        <v>191</v>
+      </c>
+      <c r="F28" s="1">
         <v>45933</v>
       </c>
-      <c r="F28" s="1">
+      <c r="G28" s="1">
         <v>45935</v>
       </c>
-      <c r="G28" t="s">
-        <v>158</v>
-      </c>
-      <c r="O28" s="1"/>
+      <c r="H28" t="s">
+        <v>157</v>
+      </c>
+      <c r="I28" t="s">
+        <v>1</v>
+      </c>
+      <c r="J28" t="s">
+        <v>136</v>
+      </c>
+      <c r="L28" s="5">
+        <v>0</v>
+      </c>
+      <c r="M28" t="s">
+        <v>191</v>
+      </c>
+      <c r="N28" t="s">
+        <v>139</v>
+      </c>
+      <c r="O28" t="s">
+        <v>2</v>
+      </c>
       <c r="P28" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q28" s="2"/>
-    </row>
-    <row r="29" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q28" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R28" s="2"/>
+    </row>
+    <row r="29" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C29" t="s">
         <v>102</v>
       </c>
       <c r="D29" t="s">
         <v>48</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" t="s">
+        <v>200</v>
+      </c>
+      <c r="F29" s="1">
         <v>45941</v>
       </c>
-      <c r="F29" s="1">
+      <c r="G29" s="1">
         <v>45945</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>36</v>
       </c>
-      <c r="H29" t="s">
-        <v>1</v>
-      </c>
       <c r="I29" t="s">
+        <v>1</v>
+      </c>
+      <c r="J29" t="s">
         <v>130</v>
       </c>
-      <c r="K29" s="5">
+      <c r="L29" s="5">
         <v>4</v>
       </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>48</v>
       </c>
-      <c r="M29" t="s">
-        <v>139</v>
-      </c>
-      <c r="N29" t="s">
-        <v>2</v>
-      </c>
-      <c r="O29" s="1" t="s">
-        <v>139</v>
+      <c r="N29" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O29" t="s">
+        <v>2</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>180</v>
+        <v>138</v>
+      </c>
+      <c r="Q29" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="R29" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="S29" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="30" spans="3:19" x14ac:dyDescent="0.2">
+        <v>225</v>
+      </c>
+      <c r="T29" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="30" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C30" t="s">
         <v>103</v>
       </c>
       <c r="D30" t="s">
         <v>62</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" t="s">
+        <v>201</v>
+      </c>
+      <c r="F30" s="1">
         <v>45986</v>
       </c>
-      <c r="F30" s="1">
+      <c r="G30" s="1">
         <v>45991</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>121</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>120</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>135</v>
       </c>
-      <c r="K30" s="5">
-        <v>2</v>
-      </c>
-      <c r="L30" t="s">
+      <c r="L30" s="5">
+        <v>2</v>
+      </c>
+      <c r="M30" t="s">
         <v>62</v>
       </c>
-      <c r="M30" t="s">
-        <v>139</v>
-      </c>
-      <c r="N30" t="s">
-        <v>2</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>139</v>
+      <c r="N30" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O30" t="s">
+        <v>2</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q30" s="2"/>
-    </row>
-    <row r="31" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q30" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R30" s="2"/>
+    </row>
+    <row r="31" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C31" t="s">
         <v>104</v>
       </c>
       <c r="D31" t="s">
         <v>55</v>
       </c>
-      <c r="E31" s="1">
-        <v>45997</v>
+      <c r="E31" t="s">
+        <v>202</v>
       </c>
       <c r="F31" s="1">
         <v>45997</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="1">
+        <v>45997</v>
+      </c>
+      <c r="H31" t="s">
         <v>38</v>
       </c>
-      <c r="H31" t="s">
-        <v>1</v>
-      </c>
       <c r="I31" t="s">
+        <v>1</v>
+      </c>
+      <c r="J31" t="s">
         <v>131</v>
       </c>
-      <c r="K31" s="5">
-        <v>2</v>
-      </c>
-      <c r="L31" t="s">
+      <c r="L31" s="5">
+        <v>2</v>
+      </c>
+      <c r="M31" t="s">
         <v>55</v>
       </c>
-      <c r="M31" t="s">
-        <v>140</v>
-      </c>
-      <c r="N31" t="s">
-        <v>2</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>139</v>
+      <c r="N31" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O31" t="s">
+        <v>2</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q31" s="2"/>
-    </row>
-    <row r="32" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R31" s="2"/>
+    </row>
+    <row r="32" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C32" t="s">
         <v>105</v>
       </c>
       <c r="D32" t="s">
         <v>56</v>
       </c>
-      <c r="E32" s="1">
-        <v>46004</v>
+      <c r="E32" t="s">
+        <v>192</v>
       </c>
       <c r="F32" s="1">
         <v>46004</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="1">
+        <v>46004</v>
+      </c>
+      <c r="H32" t="s">
         <v>37</v>
       </c>
-      <c r="H32" t="s">
-        <v>1</v>
-      </c>
       <c r="I32" t="s">
-        <v>138</v>
-      </c>
-      <c r="K32" s="5">
-        <v>2</v>
-      </c>
-      <c r="L32" t="s">
+        <v>1</v>
+      </c>
+      <c r="J32" t="s">
+        <v>137</v>
+      </c>
+      <c r="L32" s="5">
+        <v>2</v>
+      </c>
+      <c r="M32" t="s">
         <v>56</v>
       </c>
-      <c r="M32" t="s">
-        <v>140</v>
-      </c>
-      <c r="N32" t="s">
-        <v>2</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>139</v>
+      <c r="N32" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O32" t="s">
+        <v>2</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q32" s="2"/>
-    </row>
-    <row r="33" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R32" s="2"/>
+    </row>
+    <row r="33" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C33" t="s">
         <v>106</v>
       </c>
       <c r="D33" t="s">
-        <v>142</v>
-      </c>
-      <c r="E33" s="1">
+        <v>141</v>
+      </c>
+      <c r="E33" t="s">
+        <v>203</v>
+      </c>
+      <c r="F33" s="1">
         <v>46010</v>
       </c>
-      <c r="F33" s="1">
+      <c r="G33" s="1">
         <v>46012</v>
       </c>
-      <c r="G33" t="s">
-        <v>146</v>
-      </c>
       <c r="H33" t="s">
-        <v>1</v>
+        <v>145</v>
       </c>
       <c r="I33" t="s">
+        <v>1</v>
+      </c>
+      <c r="J33" t="s">
         <v>131</v>
       </c>
-      <c r="K33" s="5">
+      <c r="L33" s="5">
         <v>4</v>
       </c>
-      <c r="L33" t="s">
-        <v>142</v>
-      </c>
       <c r="M33" t="s">
-        <v>139</v>
-      </c>
-      <c r="N33" t="s">
-        <v>2</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O33" t="s">
+        <v>2</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q33" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="R33" t="s">
-        <v>175</v>
+        <v>138</v>
+      </c>
+      <c r="Q33" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R33" s="2" t="s">
+        <v>217</v>
       </c>
       <c r="S33" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="34" spans="3:19" x14ac:dyDescent="0.2">
+        <v>226</v>
+      </c>
+      <c r="T33" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="34" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C34" t="s">
         <v>107</v>
       </c>
       <c r="D34" t="s">
         <v>57</v>
       </c>
-      <c r="E34" s="1">
-        <v>46019</v>
+      <c r="E34" t="s">
+        <v>204</v>
       </c>
       <c r="F34" s="1">
         <v>46019</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34" s="1">
+        <v>46019</v>
+      </c>
+      <c r="H34" t="s">
         <v>38</v>
       </c>
-      <c r="H34" t="s">
-        <v>1</v>
-      </c>
       <c r="I34" t="s">
+        <v>1</v>
+      </c>
+      <c r="J34" t="s">
         <v>131</v>
       </c>
-      <c r="K34" s="5">
-        <v>2</v>
-      </c>
-      <c r="L34" t="s">
+      <c r="L34" s="5">
+        <v>2</v>
+      </c>
+      <c r="M34" t="s">
         <v>57</v>
       </c>
-      <c r="M34" t="s">
-        <v>140</v>
-      </c>
-      <c r="N34" t="s">
-        <v>2</v>
-      </c>
-      <c r="O34" s="1" t="s">
-        <v>139</v>
+      <c r="N34" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O34" t="s">
+        <v>2</v>
       </c>
       <c r="P34" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q34" s="2"/>
-    </row>
-    <row r="35" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q34" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R34" s="2"/>
+    </row>
+    <row r="35" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C35" t="s">
         <v>108</v>
       </c>
       <c r="D35" t="s">
         <v>58</v>
       </c>
-      <c r="E35" s="1">
-        <v>46021</v>
+      <c r="E35" t="s">
+        <v>205</v>
       </c>
       <c r="F35" s="1">
         <v>46021</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" s="1">
+        <v>46021</v>
+      </c>
+      <c r="H35" t="s">
         <v>21</v>
       </c>
-      <c r="H35" t="s">
-        <v>1</v>
-      </c>
       <c r="I35" t="s">
+        <v>1</v>
+      </c>
+      <c r="J35" t="s">
         <v>131</v>
       </c>
-      <c r="K35" s="5">
-        <v>2</v>
-      </c>
-      <c r="L35" t="s">
+      <c r="L35" s="5">
+        <v>2</v>
+      </c>
+      <c r="M35" t="s">
         <v>58</v>
       </c>
-      <c r="M35" t="s">
-        <v>140</v>
-      </c>
-      <c r="N35" t="s">
-        <v>2</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>139</v>
+      <c r="N35" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O35" t="s">
+        <v>2</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q35" s="2"/>
-    </row>
-    <row r="36" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q35" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R35" s="2"/>
+    </row>
+    <row r="36" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C36" t="s">
         <v>109</v>
       </c>
       <c r="D36" t="s">
         <v>60</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" t="s">
+        <v>206</v>
+      </c>
+      <c r="F36" s="1">
         <v>46028</v>
       </c>
-      <c r="F36" s="1">
+      <c r="G36" s="1">
         <v>46032</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>39</v>
       </c>
-      <c r="H36" t="s">
-        <v>1</v>
-      </c>
       <c r="I36" t="s">
+        <v>1</v>
+      </c>
+      <c r="J36" t="s">
         <v>135</v>
       </c>
-      <c r="K36" s="5">
+      <c r="L36" s="5">
         <v>4</v>
       </c>
-      <c r="L36" t="s">
+      <c r="M36" t="s">
         <v>60</v>
       </c>
-      <c r="M36" t="s">
-        <v>140</v>
-      </c>
-      <c r="N36" t="s">
-        <v>2</v>
-      </c>
-      <c r="O36" s="1" t="s">
-        <v>139</v>
+      <c r="N36" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O36" t="s">
+        <v>2</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q36" s="2"/>
-    </row>
-    <row r="37" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R36" s="2"/>
+    </row>
+    <row r="37" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C37" t="s">
         <v>110</v>
       </c>
       <c r="D37" t="s">
         <v>63</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" t="s">
+        <v>208</v>
+      </c>
+      <c r="F37" s="1">
         <v>46038</v>
       </c>
-      <c r="F37" s="1">
+      <c r="G37" s="1">
         <v>46041</v>
       </c>
-      <c r="G37" t="s">
-        <v>147</v>
-      </c>
       <c r="H37" t="s">
+        <v>146</v>
+      </c>
+      <c r="I37" t="s">
         <v>120</v>
       </c>
-      <c r="I37" t="s">
+      <c r="J37" t="s">
         <v>133</v>
       </c>
-      <c r="K37" s="5">
+      <c r="L37" s="5">
         <v>4</v>
       </c>
-      <c r="L37" t="s">
+      <c r="M37" t="s">
         <v>63</v>
       </c>
-      <c r="M37" t="s">
-        <v>139</v>
-      </c>
-      <c r="N37" t="s">
-        <v>2</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>139</v>
+      <c r="N37" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O37" t="s">
+        <v>2</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q37" s="2"/>
-    </row>
-    <row r="38" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q37" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R37" s="2"/>
+    </row>
+    <row r="38" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C38" t="s">
         <v>111</v>
       </c>
       <c r="D38" t="s">
         <v>64</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38" t="s">
+        <v>64</v>
+      </c>
+      <c r="F38" s="1">
         <v>46064</v>
       </c>
-      <c r="F38" s="1">
+      <c r="G38" s="1">
         <v>46069</v>
       </c>
-      <c r="G38" t="s">
-        <v>144</v>
-      </c>
       <c r="H38" t="s">
-        <v>1</v>
+        <v>143</v>
       </c>
       <c r="I38" t="s">
+        <v>1</v>
+      </c>
+      <c r="J38" t="s">
         <v>135</v>
       </c>
-      <c r="K38" s="5">
+      <c r="L38" s="5">
         <v>5</v>
       </c>
-      <c r="L38" t="s">
+      <c r="M38" t="s">
         <v>64</v>
       </c>
-      <c r="M38" t="s">
-        <v>139</v>
-      </c>
-      <c r="N38" t="s">
-        <v>2</v>
-      </c>
-      <c r="O38" s="1" t="s">
-        <v>139</v>
+      <c r="N38" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O38" t="s">
+        <v>2</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q38" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="R38" t="s">
-        <v>182</v>
+        <v>138</v>
+      </c>
+      <c r="Q38" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R38" s="2" t="s">
+        <v>170</v>
       </c>
       <c r="S38" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="39" spans="3:19" x14ac:dyDescent="0.2">
+        <v>227</v>
+      </c>
+      <c r="T38" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="39" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C39" t="s">
         <v>112</v>
       </c>
       <c r="D39" t="s">
         <v>65</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39" t="s">
+        <v>209</v>
+      </c>
+      <c r="F39" s="1">
         <v>46073</v>
       </c>
-      <c r="F39" s="1">
+      <c r="G39" s="1">
         <v>46075</v>
       </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
         <v>40</v>
       </c>
-      <c r="H39" t="s">
-        <v>1</v>
-      </c>
       <c r="I39" t="s">
+        <v>1</v>
+      </c>
+      <c r="J39" t="s">
         <v>132</v>
       </c>
-      <c r="K39" s="5">
-        <v>2</v>
-      </c>
-      <c r="L39" t="s">
+      <c r="L39" s="5">
+        <v>2</v>
+      </c>
+      <c r="M39" t="s">
         <v>65</v>
       </c>
-      <c r="M39" t="s">
-        <v>140</v>
-      </c>
-      <c r="N39" t="s">
-        <v>2</v>
-      </c>
-      <c r="O39" s="1" t="s">
-        <v>139</v>
+      <c r="N39" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O39" t="s">
+        <v>2</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q39" s="2"/>
-    </row>
-    <row r="40" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R39" s="2"/>
+    </row>
+    <row r="40" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C40" t="s">
         <v>113</v>
       </c>
       <c r="D40" t="s">
         <v>66</v>
       </c>
-      <c r="E40" s="1">
+      <c r="E40" t="s">
+        <v>210</v>
+      </c>
+      <c r="F40" s="1">
         <v>46109</v>
       </c>
-      <c r="F40" s="1">
+      <c r="G40" s="1">
         <v>46118</v>
       </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>41</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>120</v>
       </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>130</v>
       </c>
-      <c r="K40" s="5">
+      <c r="L40" s="5">
         <v>4</v>
       </c>
-      <c r="L40" t="s">
+      <c r="M40" t="s">
         <v>66</v>
       </c>
-      <c r="M40" t="s">
-        <v>139</v>
-      </c>
-      <c r="N40" t="s">
-        <v>2</v>
-      </c>
-      <c r="O40" s="1" t="s">
-        <v>139</v>
+      <c r="N40" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O40" t="s">
+        <v>2</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q40" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="R40" t="s">
-        <v>184</v>
+        <v>138</v>
+      </c>
+      <c r="Q40" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R40" s="2" t="s">
+        <v>171</v>
       </c>
       <c r="S40" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="41" spans="3:19" x14ac:dyDescent="0.2">
+        <v>228</v>
+      </c>
+      <c r="T40" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="41" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C41" t="s">
         <v>114</v>
       </c>
       <c r="D41" t="s">
         <v>67</v>
       </c>
-      <c r="E41" s="1">
-        <v>46123</v>
+      <c r="E41" t="s">
+        <v>67</v>
       </c>
       <c r="F41" s="1">
         <v>46123</v>
       </c>
-      <c r="G41" t="s">
+      <c r="G41" s="1">
+        <v>46123</v>
+      </c>
+      <c r="H41" t="s">
         <v>42</v>
       </c>
-      <c r="H41" t="s">
-        <v>1</v>
-      </c>
       <c r="I41" t="s">
+        <v>1</v>
+      </c>
+      <c r="J41" t="s">
         <v>129</v>
       </c>
-      <c r="K41" s="5">
-        <v>2</v>
-      </c>
-      <c r="L41" t="s">
+      <c r="L41" s="5">
+        <v>2</v>
+      </c>
+      <c r="M41" t="s">
         <v>67</v>
       </c>
-      <c r="M41" t="s">
-        <v>140</v>
-      </c>
-      <c r="N41" t="s">
-        <v>2</v>
-      </c>
-      <c r="O41" s="1" t="s">
-        <v>139</v>
+      <c r="N41" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O41" t="s">
+        <v>2</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q41" s="2"/>
-    </row>
-    <row r="42" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q41" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R41" s="2"/>
+    </row>
+    <row r="42" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C42" t="s">
         <v>115</v>
       </c>
       <c r="D42" t="s">
         <v>70</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E42" t="s">
+        <v>70</v>
+      </c>
+      <c r="F42" s="1">
         <v>46156</v>
       </c>
-      <c r="F42" s="1">
+      <c r="G42" s="1">
         <v>46159</v>
       </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>43</v>
       </c>
-      <c r="H42" t="s">
-        <v>1</v>
-      </c>
       <c r="I42" t="s">
+        <v>1</v>
+      </c>
+      <c r="J42" t="s">
         <v>133</v>
       </c>
-      <c r="K42" s="5">
-        <v>2</v>
-      </c>
-      <c r="L42" t="s">
+      <c r="L42" s="5">
+        <v>2</v>
+      </c>
+      <c r="M42" t="s">
         <v>70</v>
       </c>
-      <c r="M42" t="s">
-        <v>139</v>
-      </c>
-      <c r="N42" t="s">
-        <v>2</v>
-      </c>
-      <c r="O42" s="1" t="s">
-        <v>139</v>
+      <c r="N42" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O42" t="s">
+        <v>2</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q42" s="2"/>
-    </row>
-    <row r="43" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R42" s="2"/>
+    </row>
+    <row r="43" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C43" t="s">
         <v>116</v>
       </c>
       <c r="D43" t="s">
         <v>71</v>
       </c>
-      <c r="E43" s="1">
-        <v>46165</v>
+      <c r="E43" t="s">
+        <v>211</v>
       </c>
       <c r="F43" s="1">
         <v>46165</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" s="1">
+        <v>46165</v>
+      </c>
+      <c r="H43" t="s">
         <v>38</v>
       </c>
-      <c r="H43" t="s">
-        <v>1</v>
-      </c>
       <c r="I43" t="s">
+        <v>1</v>
+      </c>
+      <c r="J43" t="s">
         <v>129</v>
       </c>
-      <c r="K43" s="5">
-        <v>2</v>
-      </c>
-      <c r="L43" t="s">
+      <c r="L43" s="5">
+        <v>2</v>
+      </c>
+      <c r="M43" t="s">
         <v>71</v>
       </c>
-      <c r="M43" t="s">
-        <v>140</v>
-      </c>
-      <c r="N43" t="s">
-        <v>2</v>
-      </c>
-      <c r="O43" s="1" t="s">
-        <v>139</v>
+      <c r="N43" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O43" t="s">
+        <v>2</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q43" s="2"/>
-    </row>
-    <row r="44" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R43" s="2"/>
+    </row>
+    <row r="44" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C44" t="s">
         <v>117</v>
       </c>
       <c r="D44" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="1">
-        <v>46166</v>
+      <c r="E44" t="s">
+        <v>212</v>
       </c>
       <c r="F44" s="1">
         <v>46166</v>
       </c>
-      <c r="G44" t="s">
+      <c r="G44" s="1">
+        <v>46166</v>
+      </c>
+      <c r="H44" t="s">
         <v>20</v>
       </c>
-      <c r="H44" t="s">
-        <v>1</v>
-      </c>
       <c r="I44" t="s">
+        <v>1</v>
+      </c>
+      <c r="J44" t="s">
         <v>136</v>
       </c>
-      <c r="K44" s="5">
-        <v>2</v>
-      </c>
-      <c r="L44" t="s">
+      <c r="L44" s="5">
+        <v>2</v>
+      </c>
+      <c r="M44" t="s">
         <v>72</v>
       </c>
-      <c r="M44" t="s">
-        <v>139</v>
-      </c>
-      <c r="N44" t="s">
-        <v>2</v>
-      </c>
-      <c r="O44" s="1" t="s">
-        <v>139</v>
+      <c r="N44" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O44" t="s">
+        <v>2</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q44" s="2"/>
-    </row>
-    <row r="45" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q44" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R44" s="2"/>
+    </row>
+    <row r="45" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C45" t="s">
         <v>118</v>
       </c>
       <c r="D45" t="s">
         <v>73</v>
       </c>
-      <c r="E45" s="1">
+      <c r="E45" t="s">
+        <v>213</v>
+      </c>
+      <c r="F45" s="1">
         <v>46177</v>
       </c>
-      <c r="F45" s="1">
+      <c r="G45" s="1">
         <v>46180</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>44</v>
       </c>
-      <c r="H45" t="s">
-        <v>1</v>
-      </c>
       <c r="I45" t="s">
+        <v>1</v>
+      </c>
+      <c r="J45" t="s">
         <v>133</v>
       </c>
-      <c r="K45" s="5">
-        <v>2</v>
-      </c>
-      <c r="L45" t="s">
+      <c r="L45" s="5">
+        <v>2</v>
+      </c>
+      <c r="M45" t="s">
         <v>73</v>
       </c>
-      <c r="M45" t="s">
-        <v>139</v>
-      </c>
-      <c r="N45" t="s">
-        <v>2</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>139</v>
+      <c r="N45" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O45" t="s">
+        <v>2</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q45" s="2"/>
-    </row>
-    <row r="46" spans="3:19" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q45" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R45" s="2"/>
+    </row>
+    <row r="46" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C46" t="s">
         <v>119</v>
       </c>
       <c r="D46" t="s">
         <v>74</v>
       </c>
-      <c r="E46" s="1">
+      <c r="E46" t="s">
+        <v>74</v>
+      </c>
+      <c r="F46" s="1">
         <v>46191</v>
       </c>
-      <c r="F46" s="1">
+      <c r="G46" s="1">
         <v>46194</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>45</v>
       </c>
-      <c r="H46" t="s">
-        <v>1</v>
-      </c>
       <c r="I46" t="s">
+        <v>1</v>
+      </c>
+      <c r="J46" t="s">
         <v>133</v>
       </c>
-      <c r="K46" s="5">
-        <v>2</v>
-      </c>
-      <c r="L46" t="s">
+      <c r="L46" s="5">
+        <v>2</v>
+      </c>
+      <c r="M46" t="s">
         <v>74</v>
       </c>
-      <c r="M46" t="s">
-        <v>139</v>
-      </c>
-      <c r="N46" t="s">
-        <v>2</v>
-      </c>
-      <c r="O46" s="1" t="s">
-        <v>139</v>
+      <c r="N46" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O46" t="s">
+        <v>2</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q46" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="R46" t="s">
-        <v>186</v>
+        <v>138</v>
+      </c>
+      <c r="Q46" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R46" s="2" t="s">
+        <v>172</v>
       </c>
       <c r="S46" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="47" spans="3:19" x14ac:dyDescent="0.2">
+        <v>173</v>
+      </c>
+      <c r="T46" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="47" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C47" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D47" t="s">
         <v>75</v>
       </c>
-      <c r="E47" s="1">
+      <c r="E47" t="s">
+        <v>214</v>
+      </c>
+      <c r="F47" s="1">
         <v>46206</v>
       </c>
-      <c r="F47" s="1">
+      <c r="G47" s="1">
         <v>46215</v>
       </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>46</v>
       </c>
-      <c r="H47" t="s">
-        <v>1</v>
-      </c>
       <c r="I47" t="s">
+        <v>1</v>
+      </c>
+      <c r="J47" t="s">
         <v>130</v>
       </c>
-      <c r="K47" s="5">
+      <c r="L47" s="5">
         <v>6</v>
       </c>
-      <c r="L47" t="s">
+      <c r="M47" t="s">
         <v>75</v>
       </c>
-      <c r="M47" t="s">
-        <v>139</v>
-      </c>
-      <c r="N47" t="s">
-        <v>2</v>
-      </c>
-      <c r="O47" s="1" t="s">
-        <v>139</v>
+      <c r="N47" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O47" t="s">
+        <v>2</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q47" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="R47" t="s">
-        <v>188</v>
+        <v>138</v>
+      </c>
+      <c r="Q47" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="R47" s="2" t="s">
+        <v>174</v>
       </c>
       <c r="S47" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="48" spans="3:19" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+      <c r="T47" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="48" spans="3:20" x14ac:dyDescent="0.2">
       <c r="C48" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D48" t="s">
         <v>76</v>
       </c>
-      <c r="E48" s="1">
+      <c r="E48" t="s">
+        <v>215</v>
+      </c>
+      <c r="F48" s="1">
         <v>46220</v>
       </c>
-      <c r="F48" s="1">
+      <c r="G48" s="1">
         <v>46222</v>
       </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>47</v>
       </c>
-      <c r="H48" t="s">
-        <v>1</v>
-      </c>
       <c r="I48" t="s">
+        <v>1</v>
+      </c>
+      <c r="J48" t="s">
         <v>135</v>
       </c>
-      <c r="K48" s="5">
-        <v>2</v>
-      </c>
-      <c r="L48" t="s">
+      <c r="L48" s="5">
+        <v>2</v>
+      </c>
+      <c r="M48" t="s">
         <v>76</v>
       </c>
-      <c r="M48" t="s">
-        <v>139</v>
-      </c>
-      <c r="N48" t="s">
-        <v>2</v>
-      </c>
-      <c r="O48" s="1" t="s">
-        <v>139</v>
+      <c r="N48" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O48" t="s">
+        <v>2</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q48" s="2"/>
-    </row>
-    <row r="49" spans="3:17" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q48" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R48" s="2"/>
+    </row>
+    <row r="49" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C49" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D49" t="s">
         <v>77</v>
       </c>
-      <c r="E49" s="1">
+      <c r="E49" t="s">
+        <v>77</v>
+      </c>
+      <c r="F49" s="1">
         <v>46234</v>
       </c>
-      <c r="F49" s="1">
+      <c r="G49" s="1">
         <v>46236</v>
       </c>
-      <c r="G49" t="s">
+      <c r="H49" t="s">
         <v>78</v>
       </c>
-      <c r="H49" t="s">
-        <v>1</v>
-      </c>
       <c r="I49" t="s">
+        <v>1</v>
+      </c>
+      <c r="J49" t="s">
         <v>134</v>
       </c>
-      <c r="K49" s="5">
+      <c r="L49" s="5">
         <v>4</v>
       </c>
-      <c r="L49" t="s">
+      <c r="M49" t="s">
         <v>77</v>
       </c>
-      <c r="M49" t="s">
-        <v>139</v>
-      </c>
-      <c r="N49" t="s">
-        <v>2</v>
-      </c>
-      <c r="O49" s="1" t="s">
-        <v>139</v>
+      <c r="N49" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="O49" t="s">
+        <v>2</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q49" s="2"/>
-    </row>
-    <row r="50" spans="3:17" x14ac:dyDescent="0.2">
-      <c r="P50" s="1"/>
-      <c r="Q50" s="2"/>
-    </row>
-    <row r="51" spans="3:17" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="Q49" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="R49" s="2"/>
+    </row>
+    <row r="50" spans="3:18" x14ac:dyDescent="0.2">
+      <c r="Q50" s="1"/>
+      <c r="R50" s="2"/>
+    </row>
+    <row r="51" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C51" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C54" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C2:I2"/>
+    <mergeCell ref="C2:J2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Version 1.0 - Create privacy-safe public Travelogue build
</commit_message>
<xml_diff>
--- a/travelogue/data/Travelogue Data.xlsx
+++ b/travelogue/data/Travelogue Data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gscott/Travelogue/travelogue/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A097A26-C52F-8B42-9F09-57D8CFC541BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA03D970-B28F-FE4B-859B-1FFEDA00AF31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1900" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="239">
   <si>
     <t>Train</t>
   </si>
@@ -122,12 +122,6 @@
     <t>Ehrwald, Austria; Zugspitze, Germany</t>
   </si>
   <si>
-    <t>Missing</t>
-  </si>
-  <si>
-    <t>Rhine Mothers Day</t>
-  </si>
-  <si>
     <t>Zandvoort, Netherlands; Keukenhof, Netherlands; Bruges, Belgium; Cologne, Germany</t>
   </si>
   <si>
@@ -539,9 +533,6 @@
     <t>George's "Can't Stop Thinking About" Trip</t>
   </si>
   <si>
-    <t>Best Hotel</t>
-  </si>
-  <si>
     <t>Big Summer Trip</t>
   </si>
   <si>
@@ -629,9 +620,6 @@
     <t>Weekend in Paris</t>
   </si>
   <si>
-    <t>2025 Ski Trip with Friends</t>
-  </si>
-  <si>
     <t>Beach, Tulips, and Bruges</t>
   </si>
   <si>
@@ -695,9 +683,6 @@
     <t>A Favorite Birthday</t>
   </si>
   <si>
-    <t>Best Christmas Market Trip</t>
-  </si>
-  <si>
     <t>A big reason why we moved to Europe!</t>
   </si>
   <si>
@@ -722,19 +707,58 @@
     <t>Another bucket list country!</t>
   </si>
   <si>
-    <t>Featuring a torch-lit walk in the Black Forest.</t>
-  </si>
-  <si>
     <t>Love being citizens of the world.</t>
   </si>
   <si>
-    <t>Three wonderful countries so easy to access.</t>
-  </si>
-  <si>
-    <t>Great hikes, food, and views.</t>
-  </si>
-  <si>
     <t>Playmobil Fun Park with Cousins</t>
+  </si>
+  <si>
+    <t>TRIP-044</t>
+  </si>
+  <si>
+    <t>Netherlands Long Weekend</t>
+  </si>
+  <si>
+    <t>Most Surprising Destination</t>
+  </si>
+  <si>
+    <t>Is the Netherlands summer heaven??</t>
+  </si>
+  <si>
+    <t>IMG_6582.jpeg</t>
+  </si>
+  <si>
+    <t>Heather's Favorite Dark Horse Trip</t>
+  </si>
+  <si>
+    <t>IMG_4271.jpeg</t>
+  </si>
+  <si>
+    <t>Henry's Favorite Trip</t>
+  </si>
+  <si>
+    <t>Cows to pet, baked goods delivered to door, soccer pitch for Henry, open air museum for Heather.</t>
+  </si>
+  <si>
+    <t>Three wonderful countries you should put on your bucket list.</t>
+  </si>
+  <si>
+    <t>Great hikes, food, and views. We see why it's the "favorite place" for so many people.</t>
+  </si>
+  <si>
+    <t>Favorite Winter Weekend</t>
+  </si>
+  <si>
+    <t>Thatched roof farmhouse and three Christmas markets, one with a torch-lit walk in the Black Forest!</t>
+  </si>
+  <si>
+    <t>Nederhorst den Berg, Netherlands; Amsterdam, Netherlands</t>
+  </si>
+  <si>
+    <t>Public Summary</t>
+  </si>
+  <si>
+    <t>Public Highlight Note</t>
   </si>
 </sst>
 </file>
@@ -830,12 +854,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:T49" totalsRowShown="0">
-  <autoFilter ref="C6:T49" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C7:T49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{506FDF95-866A-4FE1-831F-816CE63DF35A}" name="Table13" displayName="Table13" ref="C6:V50" totalsRowShown="0">
+  <autoFilter ref="C6:V50" xr:uid="{39F8FA1A-A2C0-4307-92C1-B094F5EF9F16}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C7:V49">
     <sortCondition ref="F6:F49"/>
   </sortState>
-  <tableColumns count="18">
+  <tableColumns count="20">
     <tableColumn id="16" xr3:uid="{B7B8133A-8A6E-4EA5-B294-9E2634108185}" name="Trip ID"/>
     <tableColumn id="1" xr3:uid="{21A3BC19-512C-634F-86B1-18BDC46CFC75}" name="Trip Title"/>
     <tableColumn id="18" xr3:uid="{674D4376-E77D-8B47-AAE3-937EFD02E039}" name="Public Trip Title"/>
@@ -847,12 +871,14 @@
     <tableColumn id="4" xr3:uid="{2AC48918-68BC-4445-958A-BEDE9ABC901F}" name="Estimated Distance (km)"/>
     <tableColumn id="7" xr3:uid="{C60BD66D-A76F-F34B-BF2A-13F5EF0DFD45}" name="Borders Crossed" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{09CE54F5-76ED-B144-B0A1-F346A728A5F3}" name="Summary"/>
+    <tableColumn id="19" xr3:uid="{DCF6519C-DC33-804E-98DD-8EAD4E270823}" name="Public Summary"/>
     <tableColumn id="10" xr3:uid="{EE9B6364-822C-5044-A802-8D0A47DDDCF0}" name="Favorite"/>
     <tableColumn id="11" xr3:uid="{1A0019D0-FB38-3E47-B142-4DCA953885B9}" name="Status"/>
     <tableColumn id="12" xr3:uid="{FDE8B4F8-6186-E445-887C-E336131FF0FB}" name="Public"/>
     <tableColumn id="13" xr3:uid="{C973B6AD-C4FE-B340-A1BA-AFD890F06300}" name="Highlight" dataDxfId="1"/>
     <tableColumn id="14" xr3:uid="{F0452C82-0D3D-B047-9111-289C96C71818}" name="Highlight Title" dataDxfId="0"/>
     <tableColumn id="15" xr3:uid="{0E9D489D-AC48-AE4F-951A-6BF76F81E72F}" name="Highlight Note"/>
+    <tableColumn id="20" xr3:uid="{0BBD76ED-BA31-3845-BB81-9E270B61C36B}" name="Public Highlight Note"/>
     <tableColumn id="17" xr3:uid="{5E3B0C82-CFC4-354A-A772-91DB57E2EF89}" name="Photo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1179,11 +1205,11 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="C2:T54"/>
+  <dimension ref="C2:V50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="11.5" customWidth="1"/>
-    <col min="4" max="4" width="48.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.1640625" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="48.1640625" customWidth="1"/>
     <col min="6" max="6" width="11.5" customWidth="1"/>
     <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -1192,16 +1218,17 @@
     <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
     <col min="12" max="12" width="17.83203125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="48.1640625" customWidth="1"/>
-    <col min="14" max="14" width="8.83203125" customWidth="1"/>
-    <col min="15" max="15" width="10" customWidth="1"/>
-    <col min="16" max="16" width="9.33203125" customWidth="1"/>
-    <col min="17" max="17" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="31.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="49.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="48.1640625" customWidth="1"/>
+    <col min="15" max="15" width="8.83203125" customWidth="1"/>
+    <col min="16" max="16" width="10" customWidth="1"/>
+    <col min="17" max="17" width="9.33203125" customWidth="1"/>
+    <col min="18" max="18" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="49.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="49.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:20" ht="27" x14ac:dyDescent="0.35">
+    <row r="2" spans="3:22" ht="27" x14ac:dyDescent="0.35">
       <c r="C2" s="6" t="s">
         <v>9</v>
       </c>
@@ -1213,25 +1240,27 @@
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
     </row>
-    <row r="3" spans="3:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="3:22" x14ac:dyDescent="0.2">
       <c r="H3" s="4"/>
       <c r="I3" s="3"/>
       <c r="M3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="Q3" s="2"/>
-    </row>
-    <row r="4" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="N3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="R3" s="2"/>
+    </row>
+    <row r="4" spans="3:22" x14ac:dyDescent="0.2">
       <c r="M4" s="2"/>
-    </row>
-    <row r="6" spans="3:20" x14ac:dyDescent="0.2">
+      <c r="N4" s="2"/>
+    </row>
+    <row r="6" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F6" t="s">
         <v>5</v>
@@ -1249,45 +1278,51 @@
         <v>18</v>
       </c>
       <c r="K6" t="s">
+        <v>120</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="M6" t="s">
         <v>122</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="N6" t="s">
+        <v>237</v>
+      </c>
+      <c r="O6" t="s">
         <v>123</v>
       </c>
-      <c r="M6" t="s">
+      <c r="P6" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q6" t="s">
         <v>124</v>
       </c>
-      <c r="N6" t="s">
-        <v>125</v>
-      </c>
-      <c r="O6" t="s">
-        <v>8</v>
-      </c>
-      <c r="P6" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
+        <v>145</v>
+      </c>
+      <c r="S6" t="s">
+        <v>146</v>
+      </c>
+      <c r="T6" t="s">
+        <v>156</v>
+      </c>
+      <c r="U6" t="s">
+        <v>238</v>
+      </c>
+      <c r="V6" t="s">
         <v>147</v>
       </c>
-      <c r="R6" t="s">
-        <v>148</v>
-      </c>
-      <c r="S6" t="s">
-        <v>158</v>
-      </c>
-      <c r="T6" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="7" spans="3:20" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F7" s="1">
         <v>45535</v>
@@ -1302,37 +1337,40 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L7" s="5">
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>68</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O7" t="s">
-        <v>2</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>138</v>
+        <v>66</v>
+      </c>
+      <c r="N7" t="s">
+        <v>66</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P7" t="s">
+        <v>2</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R7" s="2"/>
-    </row>
-    <row r="8" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S7" s="2"/>
+    </row>
+    <row r="8" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F8" s="1">
         <v>45556</v>
@@ -1341,43 +1379,46 @@
         <v>45556</v>
       </c>
       <c r="H8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I8" t="s">
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L8" s="5">
         <v>2</v>
       </c>
       <c r="M8" t="s">
-        <v>69</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O8" t="s">
-        <v>2</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>138</v>
+        <v>67</v>
+      </c>
+      <c r="N8" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P8" t="s">
+        <v>2</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R8" s="2"/>
-    </row>
-    <row r="9" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S8" s="2"/>
+    </row>
+    <row r="9" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F9" s="1">
         <v>45592</v>
@@ -1386,51 +1427,57 @@
         <v>45595</v>
       </c>
       <c r="H9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I9" t="s">
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L9" s="5">
         <v>6</v>
       </c>
       <c r="M9" t="s">
-        <v>49</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O9" t="s">
-        <v>2</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>138</v>
+        <v>47</v>
+      </c>
+      <c r="N9" t="s">
+        <v>190</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P9" t="s">
+        <v>2</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="S9" t="s">
-        <v>159</v>
+        <v>136</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>160</v>
       </c>
       <c r="T9" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="10" spans="3:20" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+      <c r="U9" t="s">
+        <v>157</v>
+      </c>
+      <c r="V9" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F10" s="1">
         <v>45640</v>
@@ -1445,37 +1492,40 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L10" s="5">
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>50</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O10" t="s">
-        <v>2</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>138</v>
+        <v>48</v>
+      </c>
+      <c r="N10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P10" t="s">
+        <v>2</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R10" s="2"/>
-    </row>
-    <row r="11" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S10" s="2"/>
+    </row>
+    <row r="11" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F11" s="1">
         <v>45654</v>
@@ -1490,37 +1540,40 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L11" s="5">
         <v>2</v>
       </c>
       <c r="M11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="N11" t="s">
-        <v>139</v>
+        <v>49</v>
       </c>
       <c r="O11" t="s">
-        <v>2</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
+      </c>
+      <c r="P11" t="s">
+        <v>2</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R11" s="2"/>
-    </row>
-    <row r="12" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S11" s="2"/>
+    </row>
+    <row r="12" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F12" s="1">
         <v>45667</v>
@@ -1535,45 +1588,51 @@
         <v>0</v>
       </c>
       <c r="J12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L12" s="5">
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>59</v>
-      </c>
-      <c r="N12" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O12" t="s">
-        <v>2</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>138</v>
+        <v>57</v>
+      </c>
+      <c r="N12" t="s">
+        <v>191</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P12" t="s">
+        <v>2</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R12" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="S12" t="s">
-        <v>160</v>
+        <v>136</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>212</v>
       </c>
       <c r="T12" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="13" spans="3:20" x14ac:dyDescent="0.2">
+        <v>158</v>
+      </c>
+      <c r="U12" t="s">
+        <v>158</v>
+      </c>
+      <c r="V12" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="13" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="F13" s="1">
         <v>45674</v>
@@ -1588,37 +1647,40 @@
         <v>3</v>
       </c>
       <c r="J13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L13" s="5">
         <v>2</v>
       </c>
       <c r="M13" t="s">
-        <v>52</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O13" t="s">
-        <v>2</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>138</v>
+        <v>50</v>
+      </c>
+      <c r="N13" t="s">
+        <v>203</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P13" t="s">
+        <v>2</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R13" s="2"/>
-    </row>
-    <row r="14" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S13" s="2"/>
+    </row>
+    <row r="14" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F14" s="1">
         <v>45705</v>
@@ -1627,43 +1689,46 @@
         <v>45705</v>
       </c>
       <c r="H14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I14" t="s">
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L14" s="5">
         <v>2</v>
       </c>
       <c r="M14" t="s">
-        <v>53</v>
-      </c>
-      <c r="N14" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O14" t="s">
-        <v>2</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>138</v>
+        <v>51</v>
+      </c>
+      <c r="N14" t="s">
+        <v>51</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P14" t="s">
+        <v>2</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R14" s="2"/>
-    </row>
-    <row r="15" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S14" s="2"/>
+    </row>
+    <row r="15" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E15" t="s">
-        <v>195</v>
+        <v>51</v>
       </c>
       <c r="F15" s="1">
         <v>45711</v>
@@ -1678,45 +1743,51 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L15" s="5">
         <v>4</v>
       </c>
       <c r="M15" t="s">
-        <v>61</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O15" t="s">
-        <v>2</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>138</v>
+        <v>59</v>
+      </c>
+      <c r="N15" t="s">
+        <v>51</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P15" t="s">
+        <v>2</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="S15" t="s">
-        <v>218</v>
+        <v>136</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>161</v>
       </c>
       <c r="T15" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="16" spans="3:20" x14ac:dyDescent="0.2">
+        <v>213</v>
+      </c>
+      <c r="U15" t="s">
+        <v>213</v>
+      </c>
+      <c r="V15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="16" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C16" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="F16" s="1">
         <v>45765</v>
@@ -1725,13 +1796,13 @@
         <v>45768</v>
       </c>
       <c r="H16" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I16" t="s">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L16" s="5">
         <v>3</v>
@@ -1739,29 +1810,32 @@
       <c r="M16" t="s">
         <v>11</v>
       </c>
-      <c r="N16" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O16" t="s">
-        <v>2</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>138</v>
+      <c r="N16" t="s">
+        <v>192</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P16" t="s">
+        <v>2</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R16" s="2"/>
-    </row>
-    <row r="17" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S16" s="2"/>
+    </row>
+    <row r="17" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F17" s="1">
         <v>45787</v>
@@ -1776,7 +1850,7 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="L17" s="5">
         <v>2</v>
@@ -1784,23 +1858,26 @@
       <c r="M17" t="s">
         <v>12</v>
       </c>
-      <c r="N17" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O17" t="s">
-        <v>2</v>
-      </c>
-      <c r="P17" s="1" t="s">
-        <v>138</v>
+      <c r="N17" t="s">
+        <v>193</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P17" t="s">
+        <v>2</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R17" s="2"/>
-    </row>
-    <row r="18" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S17" s="2"/>
+    </row>
+    <row r="18" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D18" t="s">
         <v>13</v>
@@ -1815,13 +1892,13 @@
         <v>45809</v>
       </c>
       <c r="H18" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I18" t="s">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L18" s="5">
         <v>7</v>
@@ -1829,37 +1906,43 @@
       <c r="M18" t="s">
         <v>13</v>
       </c>
-      <c r="N18" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O18" t="s">
-        <v>2</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>138</v>
+      <c r="N18" t="s">
+        <v>13</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P18" t="s">
+        <v>2</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R18" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="S18" t="s">
-        <v>220</v>
+        <v>136</v>
+      </c>
+      <c r="R18" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>162</v>
       </c>
       <c r="T18" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="19" spans="3:20" x14ac:dyDescent="0.2">
+        <v>215</v>
+      </c>
+      <c r="U18" t="s">
+        <v>215</v>
+      </c>
+      <c r="V18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="19" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C19" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F19" s="1">
         <v>45814</v>
@@ -1868,45 +1951,51 @@
         <v>45817</v>
       </c>
       <c r="H19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I19" t="s">
         <v>3</v>
       </c>
       <c r="J19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L19" s="5">
         <v>2</v>
       </c>
       <c r="M19" t="s">
-        <v>54</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O19" t="s">
-        <v>2</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>138</v>
+        <v>52</v>
+      </c>
+      <c r="N19" t="s">
+        <v>52</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P19" t="s">
+        <v>2</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R19" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="S19" t="s">
-        <v>221</v>
+        <v>136</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>165</v>
       </c>
       <c r="T19" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="20" spans="3:20" x14ac:dyDescent="0.2">
+        <v>216</v>
+      </c>
+      <c r="U19" t="s">
+        <v>216</v>
+      </c>
+      <c r="V19" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="20" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C20" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D20" t="s">
         <v>14</v>
@@ -1921,13 +2010,13 @@
         <v>45844</v>
       </c>
       <c r="H20" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I20" t="s">
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L20" s="5">
         <v>4</v>
@@ -1935,23 +2024,37 @@
       <c r="M20" t="s">
         <v>14</v>
       </c>
-      <c r="N20" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O20" t="s">
-        <v>2</v>
-      </c>
-      <c r="P20" s="1" t="s">
-        <v>138</v>
+      <c r="N20" t="s">
+        <v>14</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P20" t="s">
+        <v>2</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R20" s="2"/>
-    </row>
-    <row r="21" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R20" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="T20" t="s">
+        <v>231</v>
+      </c>
+      <c r="U20" t="s">
+        <v>231</v>
+      </c>
+      <c r="V20" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="21" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C21" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D21" t="s">
         <v>15</v>
@@ -1966,13 +2069,13 @@
         <v>45857</v>
       </c>
       <c r="H21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I21" t="s">
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L21" s="5">
         <v>4</v>
@@ -1980,37 +2083,43 @@
       <c r="M21" t="s">
         <v>15</v>
       </c>
-      <c r="N21" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O21" t="s">
-        <v>2</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>138</v>
+      <c r="N21" t="s">
+        <v>15</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P21" t="s">
+        <v>2</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R21" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="S21" t="s">
-        <v>222</v>
+        <v>136</v>
+      </c>
+      <c r="R21" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S21" s="2" t="s">
+        <v>230</v>
       </c>
       <c r="T21" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="22" spans="3:20" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+      <c r="U21" t="s">
+        <v>217</v>
+      </c>
+      <c r="V21" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D22" t="s">
         <v>16</v>
       </c>
       <c r="E22" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="F22" s="1">
         <v>45862</v>
@@ -2019,13 +2128,13 @@
         <v>45865</v>
       </c>
       <c r="H22" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I22" t="s">
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L22" s="5">
         <v>6</v>
@@ -2033,37 +2142,43 @@
       <c r="M22" t="s">
         <v>16</v>
       </c>
-      <c r="N22" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O22" t="s">
-        <v>2</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>138</v>
+      <c r="N22" t="s">
+        <v>194</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P22" t="s">
+        <v>2</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R22" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="S22" t="s">
-        <v>219</v>
+        <v>136</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S22" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="T22" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="23" spans="3:20" x14ac:dyDescent="0.2">
+        <v>214</v>
+      </c>
+      <c r="U22" t="s">
+        <v>214</v>
+      </c>
+      <c r="V22" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D23" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E23" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F23" s="1">
         <v>45870</v>
@@ -2072,7 +2187,7 @@
         <v>45872</v>
       </c>
       <c r="H23" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I23" t="s">
         <v>1</v>
@@ -2084,31 +2199,34 @@
         <v>0</v>
       </c>
       <c r="M23" t="s">
-        <v>156</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O23" t="s">
-        <v>2</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>138</v>
+        <v>154</v>
+      </c>
+      <c r="N23" t="s">
+        <v>154</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P23" t="s">
+        <v>2</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R23" s="2"/>
-    </row>
-    <row r="24" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R23" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S23" s="2"/>
+    </row>
+    <row r="24" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C24" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D24" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E24" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F24" s="1">
         <v>45877</v>
@@ -2117,37 +2235,40 @@
         <v>45879</v>
       </c>
       <c r="H24" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I24" t="s">
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L24" s="5">
         <v>0</v>
       </c>
       <c r="M24" t="s">
-        <v>230</v>
-      </c>
-      <c r="N24" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O24" t="s">
-        <v>2</v>
-      </c>
-      <c r="P24" s="1" t="s">
-        <v>138</v>
+        <v>222</v>
+      </c>
+      <c r="N24" t="s">
+        <v>152</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P24" t="s">
+        <v>2</v>
       </c>
       <c r="Q24" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R24" s="2"/>
-    </row>
-    <row r="25" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S24" s="2"/>
+    </row>
+    <row r="25" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C25" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D25" t="s">
         <v>17</v>
@@ -2162,13 +2283,13 @@
         <v>45890</v>
       </c>
       <c r="H25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I25" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J25" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L25" s="5">
         <v>2</v>
@@ -2176,37 +2297,43 @@
       <c r="M25" t="s">
         <v>17</v>
       </c>
-      <c r="N25" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O25" t="s">
-        <v>2</v>
-      </c>
-      <c r="P25" s="1" t="s">
-        <v>138</v>
+      <c r="N25" t="s">
+        <v>17</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P25" t="s">
+        <v>2</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R25" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="S25" t="s">
-        <v>223</v>
+        <v>136</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S25" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="T25" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="26" spans="3:20" x14ac:dyDescent="0.2">
+        <v>218</v>
+      </c>
+      <c r="U25" t="s">
+        <v>218</v>
+      </c>
+      <c r="V25" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="26" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C26" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D26" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E26" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F26" s="1">
         <v>45905</v>
@@ -2215,51 +2342,57 @@
         <v>45907</v>
       </c>
       <c r="H26" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I26" t="s">
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="L26" s="5">
         <v>4</v>
       </c>
       <c r="M26" t="s">
-        <v>34</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O26" t="s">
-        <v>2</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>138</v>
+        <v>32</v>
+      </c>
+      <c r="N26" t="s">
+        <v>142</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P26" t="s">
+        <v>2</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R26" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="S26" t="s">
-        <v>224</v>
+        <v>136</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S26" s="2" t="s">
+        <v>164</v>
       </c>
       <c r="T26" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="27" spans="3:20" x14ac:dyDescent="0.2">
+        <v>219</v>
+      </c>
+      <c r="U26" t="s">
+        <v>219</v>
+      </c>
+      <c r="V26" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="27" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D27" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="F27" s="1">
         <v>45925</v>
@@ -2280,31 +2413,34 @@
         <v>2</v>
       </c>
       <c r="M27" t="s">
-        <v>35</v>
-      </c>
-      <c r="N27" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O27" t="s">
-        <v>2</v>
-      </c>
-      <c r="P27" s="1" t="s">
-        <v>138</v>
+        <v>33</v>
+      </c>
+      <c r="N27" t="s">
+        <v>195</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P27" t="s">
+        <v>2</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R27" s="2"/>
-    </row>
-    <row r="28" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R27" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S27" s="2"/>
+    </row>
+    <row r="28" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C28" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D28" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E28" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F28" s="1">
         <v>45933</v>
@@ -2313,43 +2449,46 @@
         <v>45935</v>
       </c>
       <c r="H28" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="I28" t="s">
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="L28" s="5">
         <v>0</v>
       </c>
       <c r="M28" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="N28" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="O28" t="s">
-        <v>2</v>
-      </c>
-      <c r="P28" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
+      </c>
+      <c r="P28" t="s">
+        <v>2</v>
       </c>
       <c r="Q28" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R28" s="2"/>
-    </row>
-    <row r="29" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R28" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S28" s="2"/>
+    </row>
+    <row r="29" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C29" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D29" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E29" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F29" s="1">
         <v>45941</v>
@@ -2358,51 +2497,57 @@
         <v>45945</v>
       </c>
       <c r="H29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I29" t="s">
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L29" s="5">
         <v>4</v>
       </c>
       <c r="M29" t="s">
-        <v>48</v>
-      </c>
-      <c r="N29" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O29" t="s">
-        <v>2</v>
-      </c>
-      <c r="P29" s="1" t="s">
-        <v>138</v>
+        <v>46</v>
+      </c>
+      <c r="N29" t="s">
+        <v>196</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P29" t="s">
+        <v>2</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R29" t="s">
-        <v>169</v>
+        <v>136</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="S29" t="s">
-        <v>225</v>
+        <v>166</v>
       </c>
       <c r="T29" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="30" spans="3:20" x14ac:dyDescent="0.2">
+        <v>220</v>
+      </c>
+      <c r="U29" t="s">
+        <v>220</v>
+      </c>
+      <c r="V29" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="30" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C30" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D30" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E30" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F30" s="1">
         <v>45986</v>
@@ -2411,43 +2556,46 @@
         <v>45991</v>
       </c>
       <c r="H30" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I30" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J30" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L30" s="5">
         <v>2</v>
       </c>
       <c r="M30" t="s">
-        <v>62</v>
-      </c>
-      <c r="N30" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O30" t="s">
-        <v>2</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>138</v>
+        <v>60</v>
+      </c>
+      <c r="N30" t="s">
+        <v>197</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P30" t="s">
+        <v>2</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R30" s="2"/>
-    </row>
-    <row r="31" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S30" s="2"/>
+    </row>
+    <row r="31" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C31" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E31" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F31" s="1">
         <v>45997</v>
@@ -2456,43 +2604,46 @@
         <v>45997</v>
       </c>
       <c r="H31" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I31" t="s">
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L31" s="5">
         <v>2</v>
       </c>
       <c r="M31" t="s">
-        <v>55</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O31" t="s">
-        <v>2</v>
-      </c>
-      <c r="P31" s="1" t="s">
-        <v>138</v>
+        <v>53</v>
+      </c>
+      <c r="N31" t="s">
+        <v>198</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P31" t="s">
+        <v>2</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R31" s="2"/>
-    </row>
-    <row r="32" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R31" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S31" s="2"/>
+    </row>
+    <row r="32" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C32" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D32" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E32" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F32" s="1">
         <v>46004</v>
@@ -2501,43 +2652,46 @@
         <v>46004</v>
       </c>
       <c r="H32" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I32" t="s">
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="L32" s="5">
         <v>2</v>
       </c>
       <c r="M32" t="s">
-        <v>56</v>
-      </c>
-      <c r="N32" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N32" t="s">
+        <v>189</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P32" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="R32" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S32" s="2"/>
+    </row>
+    <row r="33" spans="3:22" x14ac:dyDescent="0.2">
+      <c r="C33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" t="s">
         <v>139</v>
       </c>
-      <c r="O32" t="s">
-        <v>2</v>
-      </c>
-      <c r="P32" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R32" s="2"/>
-    </row>
-    <row r="33" spans="3:20" x14ac:dyDescent="0.2">
-      <c r="C33" t="s">
-        <v>106</v>
-      </c>
-      <c r="D33" t="s">
-        <v>141</v>
-      </c>
       <c r="E33" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F33" s="1">
         <v>46010</v>
@@ -2546,51 +2700,57 @@
         <v>46012</v>
       </c>
       <c r="H33" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I33" t="s">
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L33" s="5">
         <v>4</v>
       </c>
       <c r="M33" t="s">
-        <v>141</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O33" t="s">
-        <v>2</v>
-      </c>
-      <c r="P33" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
+      </c>
+      <c r="N33" t="s">
+        <v>199</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P33" t="s">
+        <v>2</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R33" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="S33" t="s">
-        <v>226</v>
+        <v>136</v>
+      </c>
+      <c r="R33" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S33" s="2" t="s">
+        <v>234</v>
       </c>
       <c r="T33" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="34" spans="3:20" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+      <c r="U33" t="s">
+        <v>235</v>
+      </c>
+      <c r="V33" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="34" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C34" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D34" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E34" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="F34" s="1">
         <v>46019</v>
@@ -2599,43 +2759,46 @@
         <v>46019</v>
       </c>
       <c r="H34" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I34" t="s">
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L34" s="5">
         <v>2</v>
       </c>
       <c r="M34" t="s">
-        <v>57</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O34" t="s">
-        <v>2</v>
-      </c>
-      <c r="P34" s="1" t="s">
-        <v>138</v>
+        <v>55</v>
+      </c>
+      <c r="N34" t="s">
+        <v>200</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P34" t="s">
+        <v>2</v>
       </c>
       <c r="Q34" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R34" s="2"/>
-    </row>
-    <row r="35" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R34" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S34" s="2"/>
+    </row>
+    <row r="35" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C35" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D35" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E35" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="F35" s="1">
         <v>46021</v>
@@ -2650,37 +2813,40 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="L35" s="5">
         <v>2</v>
       </c>
       <c r="M35" t="s">
+        <v>56</v>
+      </c>
+      <c r="N35" t="s">
+        <v>201</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P35" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q35" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="R35" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S35" s="2"/>
+    </row>
+    <row r="36" spans="3:22" x14ac:dyDescent="0.2">
+      <c r="C36" t="s">
+        <v>107</v>
+      </c>
+      <c r="D36" t="s">
         <v>58</v>
       </c>
-      <c r="N35" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O35" t="s">
-        <v>2</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R35" s="2"/>
-    </row>
-    <row r="36" spans="3:20" x14ac:dyDescent="0.2">
-      <c r="C36" t="s">
-        <v>109</v>
-      </c>
-      <c r="D36" t="s">
-        <v>60</v>
-      </c>
       <c r="E36" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F36" s="1">
         <v>46028</v>
@@ -2689,43 +2855,46 @@
         <v>46032</v>
       </c>
       <c r="H36" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I36" t="s">
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L36" s="5">
         <v>4</v>
       </c>
       <c r="M36" t="s">
-        <v>60</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O36" t="s">
-        <v>2</v>
-      </c>
-      <c r="P36" s="1" t="s">
-        <v>138</v>
+        <v>58</v>
+      </c>
+      <c r="N36" t="s">
+        <v>202</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P36" t="s">
+        <v>2</v>
       </c>
       <c r="Q36" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R36" s="2"/>
-    </row>
-    <row r="37" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S36" s="2"/>
+    </row>
+    <row r="37" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C37" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D37" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E37" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F37" s="1">
         <v>46038</v>
@@ -2734,43 +2903,46 @@
         <v>46041</v>
       </c>
       <c r="H37" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I37" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J37" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L37" s="5">
         <v>4</v>
       </c>
       <c r="M37" t="s">
-        <v>63</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O37" t="s">
-        <v>2</v>
-      </c>
-      <c r="P37" s="1" t="s">
-        <v>138</v>
+        <v>61</v>
+      </c>
+      <c r="N37" t="s">
+        <v>204</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P37" t="s">
+        <v>2</v>
       </c>
       <c r="Q37" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R37" s="2"/>
-    </row>
-    <row r="38" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R37" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S37" s="2"/>
+    </row>
+    <row r="38" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C38" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E38" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F38" s="1">
         <v>46064</v>
@@ -2779,51 +2951,57 @@
         <v>46069</v>
       </c>
       <c r="H38" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I38" t="s">
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L38" s="5">
         <v>5</v>
       </c>
       <c r="M38" t="s">
-        <v>64</v>
-      </c>
-      <c r="N38" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O38" t="s">
-        <v>2</v>
-      </c>
-      <c r="P38" s="1" t="s">
-        <v>138</v>
+        <v>62</v>
+      </c>
+      <c r="N38" t="s">
+        <v>62</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P38" t="s">
+        <v>2</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R38" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="S38" t="s">
-        <v>227</v>
+        <v>136</v>
+      </c>
+      <c r="R38" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S38" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="T38" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="39" spans="3:20" x14ac:dyDescent="0.2">
+        <v>221</v>
+      </c>
+      <c r="U38" t="s">
+        <v>221</v>
+      </c>
+      <c r="V38" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="39" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C39" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D39" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E39" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="F39" s="1">
         <v>46073</v>
@@ -2832,43 +3010,46 @@
         <v>46075</v>
       </c>
       <c r="H39" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I39" t="s">
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L39" s="5">
         <v>2</v>
       </c>
       <c r="M39" t="s">
-        <v>65</v>
-      </c>
-      <c r="N39" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O39" t="s">
-        <v>2</v>
-      </c>
-      <c r="P39" s="1" t="s">
-        <v>138</v>
+        <v>63</v>
+      </c>
+      <c r="N39" t="s">
+        <v>205</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P39" t="s">
+        <v>2</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R39" s="2"/>
-    </row>
-    <row r="40" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R39" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S39" s="2"/>
+    </row>
+    <row r="40" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C40" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D40" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E40" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="F40" s="1">
         <v>46109</v>
@@ -2877,51 +3058,57 @@
         <v>46118</v>
       </c>
       <c r="H40" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I40" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J40" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L40" s="5">
         <v>4</v>
       </c>
       <c r="M40" t="s">
-        <v>66</v>
-      </c>
-      <c r="N40" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O40" t="s">
-        <v>2</v>
-      </c>
-      <c r="P40" s="1" t="s">
-        <v>138</v>
+        <v>64</v>
+      </c>
+      <c r="N40" t="s">
+        <v>206</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P40" t="s">
+        <v>2</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R40" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="S40" t="s">
-        <v>228</v>
+        <v>136</v>
+      </c>
+      <c r="R40" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S40" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="T40" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="41" spans="3:20" x14ac:dyDescent="0.2">
+        <v>232</v>
+      </c>
+      <c r="U40" t="s">
+        <v>232</v>
+      </c>
+      <c r="V40" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="41" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C41" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D41" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E41" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F41" s="1">
         <v>46123</v>
@@ -2930,43 +3117,46 @@
         <v>46123</v>
       </c>
       <c r="H41" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I41" t="s">
         <v>1</v>
       </c>
       <c r="J41" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="L41" s="5">
         <v>2</v>
       </c>
       <c r="M41" t="s">
-        <v>67</v>
-      </c>
-      <c r="N41" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O41" t="s">
-        <v>2</v>
-      </c>
-      <c r="P41" s="1" t="s">
-        <v>138</v>
+        <v>65</v>
+      </c>
+      <c r="N41" t="s">
+        <v>65</v>
+      </c>
+      <c r="O41" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P41" t="s">
+        <v>2</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R41" s="2"/>
-    </row>
-    <row r="42" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R41" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S41" s="2"/>
+    </row>
+    <row r="42" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C42" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D42" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E42" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F42" s="1">
         <v>46156</v>
@@ -2975,43 +3165,46 @@
         <v>46159</v>
       </c>
       <c r="H42" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I42" t="s">
         <v>1</v>
       </c>
       <c r="J42" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L42" s="5">
         <v>2</v>
       </c>
       <c r="M42" t="s">
-        <v>70</v>
-      </c>
-      <c r="N42" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O42" t="s">
-        <v>2</v>
-      </c>
-      <c r="P42" s="1" t="s">
-        <v>138</v>
+        <v>68</v>
+      </c>
+      <c r="N42" t="s">
+        <v>68</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P42" t="s">
+        <v>2</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R42" s="2"/>
-    </row>
-    <row r="43" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R42" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S42" s="2"/>
+    </row>
+    <row r="43" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C43" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D43" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E43" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F43" s="1">
         <v>46165</v>
@@ -3020,43 +3213,46 @@
         <v>46165</v>
       </c>
       <c r="H43" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I43" t="s">
         <v>1</v>
       </c>
       <c r="J43" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="L43" s="5">
         <v>2</v>
       </c>
       <c r="M43" t="s">
-        <v>71</v>
-      </c>
-      <c r="N43" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O43" t="s">
-        <v>2</v>
-      </c>
-      <c r="P43" s="1" t="s">
-        <v>138</v>
+        <v>69</v>
+      </c>
+      <c r="N43" t="s">
+        <v>207</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P43" t="s">
+        <v>2</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R43" s="2"/>
-    </row>
-    <row r="44" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R43" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S43" s="2"/>
+    </row>
+    <row r="44" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C44" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D44" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E44" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F44" s="1">
         <v>46166</v>
@@ -3071,37 +3267,40 @@
         <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="L44" s="5">
         <v>2</v>
       </c>
       <c r="M44" t="s">
-        <v>72</v>
-      </c>
-      <c r="N44" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O44" t="s">
-        <v>2</v>
-      </c>
-      <c r="P44" s="1" t="s">
-        <v>138</v>
+        <v>70</v>
+      </c>
+      <c r="N44" t="s">
+        <v>208</v>
+      </c>
+      <c r="O44" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P44" t="s">
+        <v>2</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R44" s="2"/>
-    </row>
-    <row r="45" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R44" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S44" s="2"/>
+    </row>
+    <row r="45" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C45" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D45" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E45" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F45" s="1">
         <v>46177</v>
@@ -3110,43 +3309,46 @@
         <v>46180</v>
       </c>
       <c r="H45" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I45" t="s">
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L45" s="5">
         <v>2</v>
       </c>
       <c r="M45" t="s">
-        <v>73</v>
-      </c>
-      <c r="N45" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O45" t="s">
-        <v>2</v>
-      </c>
-      <c r="P45" s="1" t="s">
-        <v>138</v>
+        <v>71</v>
+      </c>
+      <c r="N45" t="s">
+        <v>209</v>
+      </c>
+      <c r="O45" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P45" t="s">
+        <v>2</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R45" s="2"/>
-    </row>
-    <row r="46" spans="3:20" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R45" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S45" s="2"/>
+    </row>
+    <row r="46" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C46" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D46" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E46" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F46" s="1">
         <v>46191</v>
@@ -3155,51 +3357,57 @@
         <v>46194</v>
       </c>
       <c r="H46" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I46" t="s">
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L46" s="5">
         <v>2</v>
       </c>
       <c r="M46" t="s">
-        <v>74</v>
-      </c>
-      <c r="N46" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O46" t="s">
-        <v>2</v>
-      </c>
-      <c r="P46" s="1" t="s">
-        <v>138</v>
+        <v>72</v>
+      </c>
+      <c r="N46" t="s">
+        <v>72</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P46" t="s">
+        <v>2</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R46" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="S46" t="s">
-        <v>173</v>
+        <v>136</v>
+      </c>
+      <c r="R46" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S46" s="2" t="s">
+        <v>169</v>
       </c>
       <c r="T46" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="47" spans="3:20" x14ac:dyDescent="0.2">
+        <v>170</v>
+      </c>
+      <c r="U46" t="s">
+        <v>170</v>
+      </c>
+      <c r="V46" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="47" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C47" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D47" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E47" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="F47" s="1">
         <v>46206</v>
@@ -3208,51 +3416,57 @@
         <v>46215</v>
       </c>
       <c r="H47" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I47" t="s">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L47" s="5">
         <v>6</v>
       </c>
       <c r="M47" t="s">
-        <v>75</v>
-      </c>
-      <c r="N47" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="O47" t="s">
-        <v>2</v>
-      </c>
-      <c r="P47" s="1" t="s">
-        <v>138</v>
+        <v>73</v>
+      </c>
+      <c r="N47" t="s">
+        <v>210</v>
+      </c>
+      <c r="O47" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P47" t="s">
+        <v>2</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="R47" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="S47" t="s">
-        <v>229</v>
+        <v>136</v>
+      </c>
+      <c r="R47" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S47" s="2" t="s">
+        <v>171</v>
       </c>
       <c r="T47" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="48" spans="3:20" x14ac:dyDescent="0.2">
+        <v>233</v>
+      </c>
+      <c r="U47" t="s">
+        <v>233</v>
+      </c>
+      <c r="V47" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="48" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C48" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D48" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E48" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="F48" s="1">
         <v>46220</v>
@@ -3261,43 +3475,46 @@
         <v>46222</v>
       </c>
       <c r="H48" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I48" t="s">
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L48" s="5">
         <v>2</v>
       </c>
       <c r="M48" t="s">
-        <v>76</v>
-      </c>
-      <c r="N48" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O48" t="s">
-        <v>2</v>
-      </c>
-      <c r="P48" s="1" t="s">
-        <v>138</v>
+        <v>74</v>
+      </c>
+      <c r="N48" t="s">
+        <v>211</v>
+      </c>
+      <c r="O48" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P48" t="s">
+        <v>2</v>
       </c>
       <c r="Q48" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R48" s="2"/>
-    </row>
-    <row r="49" spans="3:18" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="R48" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S48" s="2"/>
+    </row>
+    <row r="49" spans="3:22" x14ac:dyDescent="0.2">
       <c r="C49" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D49" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E49" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F49" s="1">
         <v>46234</v>
@@ -3306,46 +3523,94 @@
         <v>46236</v>
       </c>
       <c r="H49" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I49" t="s">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L49" s="5">
         <v>4</v>
       </c>
       <c r="M49" t="s">
-        <v>77</v>
-      </c>
-      <c r="N49" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="O49" t="s">
-        <v>2</v>
-      </c>
-      <c r="P49" s="1" t="s">
-        <v>138</v>
+        <v>75</v>
+      </c>
+      <c r="N49" t="s">
+        <v>75</v>
+      </c>
+      <c r="O49" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="P49" t="s">
+        <v>2</v>
       </c>
       <c r="Q49" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="R49" s="2"/>
-    </row>
-    <row r="50" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="Q50" s="1"/>
-      <c r="R50" s="2"/>
-    </row>
-    <row r="51" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="C51" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="54" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="C54" t="s">
-        <v>27</v>
+        <v>136</v>
+      </c>
+      <c r="R49" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S49" s="2"/>
+    </row>
+    <row r="50" spans="3:22" x14ac:dyDescent="0.2">
+      <c r="C50" t="s">
+        <v>223</v>
+      </c>
+      <c r="D50" t="s">
+        <v>224</v>
+      </c>
+      <c r="E50" t="s">
+        <v>224</v>
+      </c>
+      <c r="F50" s="1">
+        <v>46240</v>
+      </c>
+      <c r="G50" s="1">
+        <v>46244</v>
+      </c>
+      <c r="H50" t="s">
+        <v>236</v>
+      </c>
+      <c r="I50" t="s">
+        <v>1</v>
+      </c>
+      <c r="J50" t="s">
+        <v>131</v>
+      </c>
+      <c r="L50" s="5">
+        <v>4</v>
+      </c>
+      <c r="M50" t="s">
+        <v>224</v>
+      </c>
+      <c r="N50" t="s">
+        <v>224</v>
+      </c>
+      <c r="O50" t="s">
+        <v>136</v>
+      </c>
+      <c r="P50" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>136</v>
+      </c>
+      <c r="R50" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="S50" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="T50" t="s">
+        <v>226</v>
+      </c>
+      <c r="U50" t="s">
+        <v>226</v>
+      </c>
+      <c r="V50" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Travelogue social sharing graphics
</commit_message>
<xml_diff>
--- a/travelogue/data/Travelogue Data.xlsx
+++ b/travelogue/data/Travelogue Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gscott/Travelogue/travelogue/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA03D970-B28F-FE4B-859B-1FFEDA00AF31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0730901-3AB7-1741-B32D-360C0B7F43A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1900" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="242">
   <si>
     <t>Train</t>
   </si>
@@ -728,9 +728,6 @@
     <t>IMG_6582.jpeg</t>
   </si>
   <si>
-    <t>Heather's Favorite Dark Horse Trip</t>
-  </si>
-  <si>
     <t>IMG_4271.jpeg</t>
   </si>
   <si>
@@ -759,6 +756,18 @@
   </si>
   <si>
     <t>Public Highlight Note</t>
+  </si>
+  <si>
+    <t>Heather's Favorite "Low Key" Trip</t>
+  </si>
+  <si>
+    <t>Cows to pet, baked goods delivered to door, soccer pitch for Henry, Heather's favorite open air museum.</t>
+  </si>
+  <si>
+    <t>Revisiting our favorite honeymoon spot, with our kids!</t>
+  </si>
+  <si>
+    <t>Back to Bol</t>
   </si>
 </sst>
 </file>
@@ -1287,7 +1296,7 @@
         <v>122</v>
       </c>
       <c r="N6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="O6" t="s">
         <v>123</v>
@@ -1308,7 +1317,7 @@
         <v>156</v>
       </c>
       <c r="U6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="V6" t="s">
         <v>147</v>
@@ -1966,7 +1975,7 @@
         <v>52</v>
       </c>
       <c r="N19" t="s">
-        <v>52</v>
+        <v>241</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>136</v>
@@ -1984,7 +1993,7 @@
         <v>165</v>
       </c>
       <c r="T19" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="U19" t="s">
         <v>216</v>
@@ -2040,16 +2049,16 @@
         <v>136</v>
       </c>
       <c r="S20" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="T20" t="s">
+        <v>239</v>
+      </c>
+      <c r="U20" t="s">
+        <v>230</v>
+      </c>
+      <c r="V20" t="s">
         <v>228</v>
-      </c>
-      <c r="T20" t="s">
-        <v>231</v>
-      </c>
-      <c r="U20" t="s">
-        <v>231</v>
-      </c>
-      <c r="V20" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="21" spans="3:22" x14ac:dyDescent="0.2">
@@ -2099,7 +2108,7 @@
         <v>136</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="T21" t="s">
         <v>217</v>
@@ -2730,13 +2739,13 @@
         <v>136</v>
       </c>
       <c r="S33" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="T33" t="s">
         <v>234</v>
       </c>
-      <c r="T33" t="s">
-        <v>235</v>
-      </c>
       <c r="U33" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V33" t="s">
         <v>173</v>
@@ -3091,10 +3100,10 @@
         <v>168</v>
       </c>
       <c r="T40" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="U40" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="V40" t="s">
         <v>172</v>
@@ -3449,10 +3458,10 @@
         <v>171</v>
       </c>
       <c r="T47" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="U47" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="V47" t="s">
         <v>181</v>
@@ -3571,7 +3580,7 @@
         <v>46244</v>
       </c>
       <c r="H50" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I50" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Update Travelogue trip data
</commit_message>
<xml_diff>
--- a/travelogue/data/Travelogue Data.xlsx
+++ b/travelogue/data/Travelogue Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gscott/Travelogue/travelogue/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0730901-3AB7-1741-B32D-360C0B7F43A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8DD0560-F5A3-AC46-A080-3B7441CC3425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="243">
   <si>
     <t>Train</t>
   </si>
@@ -768,6 +768,9 @@
   </si>
   <si>
     <t>Back to Bol</t>
+  </si>
+  <si>
+    <t>Austrian Skiing with Friends</t>
   </si>
 </sst>
 </file>
@@ -1761,7 +1764,7 @@
         <v>59</v>
       </c>
       <c r="N15" t="s">
-        <v>51</v>
+        <v>242</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>136</v>

</xml_diff>

<commit_message>
Update public trip titles
</commit_message>
<xml_diff>
--- a/travelogue/data/Travelogue Data.xlsx
+++ b/travelogue/data/Travelogue Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gscott/Travelogue/travelogue/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8DD0560-F5A3-AC46-A080-3B7441CC3425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E854B763-519F-5F42-A9B2-354856DC0F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="14860" xr2:uid="{3D5DA885-6A4C-4137-8B89-C9D809B8BE43}"/>
   </bookViews>
@@ -1740,7 +1740,7 @@
         <v>59</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>242</v>
       </c>
       <c r="F15" s="1">
         <v>45711</v>
@@ -1954,7 +1954,7 @@
         <v>52</v>
       </c>
       <c r="E19" t="s">
-        <v>52</v>
+        <v>241</v>
       </c>
       <c r="F19" s="1">
         <v>45814</v>

</xml_diff>